<commit_message>
modelo D con las decisiones del 29/10 (sin cuota, mínimo 300, billeteras separadas, 1% en tokens)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PW6Q8w1k9NaeArkk4QShv1
</commit_message>
<xml_diff>
--- a/docs/modelo_negocio_lloyd.xlsx
+++ b/docs/modelo_negocio_lloyd.xlsx
@@ -207,7 +207,7 @@
     <t xml:space="preserve">Comisión de ejecución por operación con tokens (todos)</t>
   </si>
   <si>
-    <t xml:space="preserve">Embebida en el precio como 'fee included'. 0,25% es lo que cobra Jupiter con integradores; los bots de Telegram cobran 0,5–1%.</t>
+    <t xml:space="preserve">Gastón 29/10: el fee encubierto es fundamental; 5–10%/mes en memecoins no es grave. 1% solo sobre operaciones con tokens ≈ 9%/mes.</t>
   </si>
   <si>
     <t xml:space="preserve">Parte del volumen que es operación con tokens (el resto es USDC/SOL)</t>
@@ -225,7 +225,7 @@
     <t xml:space="preserve">Externos · cuota de ingreso (US$), opcional</t>
   </si>
   <si>
-    <t xml:space="preserve">Se paga una vez al entrar.</t>
+    <t xml:space="preserve">Gastón 29/10: sin cuota de ingreso; la gente no va a pagar para ver cómo funciona.</t>
   </si>
   <si>
     <t xml:space="preserve">Externos · meses que cubre la cuota de ingreso</t>
@@ -240,13 +240,13 @@
     <t xml:space="preserve">La promesa: nada sobre ganancias. No tocar.</t>
   </si>
   <si>
-    <t xml:space="preserve">Gastón, 29/10: sin mínimos; la mayoría va a probar con US$100–150. Pocos van a poner US$1.000.</t>
+    <t xml:space="preserve">Gastón 29/10: mínimo de depósito US$300.</t>
   </si>
   <si>
     <t xml:space="preserve">Billetera única (ómnibus) con libro interno: 1 = sí, 0 = una billetera por usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">Con ómnibus, Lloyd ejecuta UNA transacción por decisión para todos; el costo on-chain deja de crecer con los usuarios. Es lo que hace cualquier vault o bot de Telegram.</t>
+    <t xml:space="preserve">Gastón 29/10: billeteras separadas, cada uno ve su progreso.</t>
   </si>
   <si>
     <t xml:space="preserve">Comisión de ejecución que paga cada cliente por mes (% de su capital)</t>
@@ -478,7 +478,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="8">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -486,8 +486,7 @@
     <numFmt numFmtId="168" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="169" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="170" formatCode="0.0\x"/>
-    <numFmt numFmtId="171" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
-    <numFmt numFmtId="172" formatCode="#,##0"/>
+    <numFmt numFmtId="171" formatCode="#,##0"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -630,7 +629,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="45">
+  <cellXfs count="33">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -707,55 +706,27 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="171" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -763,27 +734,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -799,15 +754,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="172" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="171" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1497,700 +1448,700 @@
   <dimension ref="A1:H34"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="60"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="19" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="20"/>
-      <c r="C1" s="20"/>
-      <c r="D1" s="20"/>
-      <c r="E1" s="20"/>
-      <c r="F1" s="20"/>
-      <c r="G1" s="20"/>
-      <c r="H1" s="20"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
+      <c r="F1" s="3"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="3"/>
     </row>
     <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="19" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="C2" s="21"/>
-      <c r="D2" s="21"/>
-      <c r="E2" s="21"/>
-      <c r="F2" s="21"/>
-      <c r="G2" s="21"/>
-      <c r="H2" s="21"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="20"/>
-      <c r="B3" s="20"/>
-      <c r="C3" s="20"/>
-      <c r="D3" s="20"/>
-      <c r="E3" s="20"/>
-      <c r="F3" s="20"/>
-      <c r="G3" s="20"/>
-      <c r="H3" s="20"/>
-    </row>
-    <row r="4" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="20" t="s">
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3"/>
+      <c r="B3" s="3"/>
+      <c r="C3" s="3"/>
+      <c r="D3" s="3"/>
+      <c r="E3" s="3"/>
+      <c r="F3" s="3"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="3"/>
+    </row>
+    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="22" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
+      <c r="B4" s="8" t="n">
+        <v>0.01</v>
+      </c>
+      <c r="C4" s="3"/>
+      <c r="D4" s="3"/>
+      <c r="E4" s="3"/>
+      <c r="F4" s="3"/>
+      <c r="G4" s="3"/>
       <c r="H4" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="20" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="22" t="n">
+      <c r="B5" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="C5" s="20"/>
-      <c r="D5" s="20"/>
-      <c r="E5" s="20"/>
-      <c r="F5" s="20"/>
-      <c r="G5" s="20"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
       <c r="H5" s="7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="20" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="B6" s="22" t="n">
+      <c r="B6" s="8" t="n">
         <v>0.2</v>
       </c>
-      <c r="C6" s="20"/>
-      <c r="D6" s="20"/>
-      <c r="E6" s="20"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
+      <c r="C6" s="3"/>
+      <c r="D6" s="3"/>
+      <c r="E6" s="3"/>
+      <c r="F6" s="3"/>
+      <c r="G6" s="3"/>
       <c r="H6" s="7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="20" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="23" t="n">
-        <v>49</v>
-      </c>
-      <c r="C7" s="20"/>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="20"/>
+      <c r="B7" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="3"/>
+      <c r="D7" s="3"/>
+      <c r="E7" s="3"/>
+      <c r="F7" s="3"/>
+      <c r="G7" s="3"/>
       <c r="H7" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="20" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="24" t="n">
+      <c r="B8" s="9" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="20"/>
-      <c r="D8" s="20"/>
-      <c r="E8" s="20"/>
-      <c r="F8" s="20"/>
-      <c r="G8" s="20"/>
+      <c r="C8" s="3"/>
+      <c r="D8" s="3"/>
+      <c r="E8" s="3"/>
+      <c r="F8" s="3"/>
+      <c r="G8" s="3"/>
       <c r="H8" s="7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="20" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B9" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="20"/>
-      <c r="D9" s="20"/>
-      <c r="E9" s="20"/>
-      <c r="F9" s="20"/>
-      <c r="G9" s="20"/>
+      <c r="B9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="3"/>
+      <c r="D9" s="3"/>
+      <c r="E9" s="3"/>
+      <c r="F9" s="3"/>
+      <c r="G9" s="3"/>
       <c r="H9" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="20" t="s">
+    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="23" t="n">
-        <v>150</v>
-      </c>
-      <c r="C10" s="20"/>
-      <c r="D10" s="20"/>
-      <c r="E10" s="20"/>
-      <c r="F10" s="20"/>
-      <c r="G10" s="20"/>
+      <c r="B10" s="12" t="n">
+        <v>300</v>
+      </c>
+      <c r="C10" s="3"/>
+      <c r="D10" s="3"/>
+      <c r="E10" s="3"/>
+      <c r="F10" s="3"/>
+      <c r="G10" s="3"/>
       <c r="H10" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="20" t="s">
+    <row r="11" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="24" t="n">
-        <v>1</v>
-      </c>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
+      <c r="B11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="3"/>
+      <c r="D11" s="3"/>
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+      <c r="G11" s="3"/>
       <c r="H11" s="7" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20"/>
-      <c r="B12" s="20"/>
-      <c r="C12" s="20"/>
-      <c r="D12" s="20"/>
-      <c r="E12" s="20"/>
-      <c r="F12" s="20"/>
-      <c r="G12" s="20"/>
-      <c r="H12" s="20"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3"/>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+      <c r="E12" s="3"/>
+      <c r="F12" s="3"/>
+      <c r="G12" s="3"/>
+      <c r="H12" s="3"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="25" t="n">
+      <c r="B13" s="20" t="n">
         <f aca="false">Supuestos!$B$40*$B$5*$B$4</f>
-        <v>0.0225</v>
-      </c>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="20" t="s">
+        <v>0.09</v>
+      </c>
+      <c r="C13" s="3"/>
+      <c r="D13" s="3"/>
+      <c r="E13" s="3"/>
+      <c r="F13" s="3"/>
+      <c r="G13" s="3"/>
+      <c r="H13" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="3" t="s">
         <v>75</v>
       </c>
-      <c r="B14" s="25" t="n">
+      <c r="B14" s="20" t="n">
         <f aca="false">Supuestos!$B$8-$B$13</f>
-        <v>0.0775</v>
-      </c>
-      <c r="C14" s="20"/>
-      <c r="D14" s="20"/>
-      <c r="E14" s="20"/>
-      <c r="F14" s="20"/>
-      <c r="G14" s="20"/>
-      <c r="H14" s="20"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="20" t="s">
+        <v>0.01</v>
+      </c>
+      <c r="C14" s="3"/>
+      <c r="D14" s="3"/>
+      <c r="E14" s="3"/>
+      <c r="F14" s="3"/>
+      <c r="G14" s="3"/>
+      <c r="H14" s="3"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="B15" s="25" t="n">
+      <c r="B15" s="20" t="n">
         <f aca="false">Supuestos!$B$8-$B$13-MAX(0,Supuestos!$B$8-$B$13)*$B$6</f>
-        <v>0.062</v>
-      </c>
-      <c r="C15" s="20"/>
-      <c r="D15" s="20"/>
-      <c r="E15" s="20"/>
-      <c r="F15" s="20"/>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="20" t="s">
+        <v>0.00800000000000001</v>
+      </c>
+      <c r="C15" s="3"/>
+      <c r="D15" s="3"/>
+      <c r="E15" s="3"/>
+      <c r="F15" s="3"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="3" t="s">
         <v>77</v>
       </c>
-      <c r="B16" s="26" t="n">
+      <c r="B16" s="21" t="n">
         <f aca="false">$B$13</f>
-        <v>0.0225</v>
-      </c>
-      <c r="C16" s="20"/>
-      <c r="D16" s="20"/>
-      <c r="E16" s="20"/>
-      <c r="F16" s="20"/>
-      <c r="G16" s="20"/>
-      <c r="H16" s="20"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="20"/>
-      <c r="B17" s="20"/>
-      <c r="C17" s="20"/>
-      <c r="D17" s="20"/>
-      <c r="E17" s="20"/>
-      <c r="F17" s="20"/>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="27" t="s">
+        <v>0.09</v>
+      </c>
+      <c r="C16" s="3"/>
+      <c r="D16" s="3"/>
+      <c r="E16" s="3"/>
+      <c r="F16" s="3"/>
+      <c r="G16" s="3"/>
+      <c r="H16" s="3"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="3"/>
+      <c r="B17" s="3"/>
+      <c r="C17" s="3"/>
+      <c r="D17" s="3"/>
+      <c r="E17" s="3"/>
+      <c r="F17" s="3"/>
+      <c r="G17" s="3"/>
+      <c r="H17" s="3"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="B18" s="20"/>
-      <c r="C18" s="20"/>
-      <c r="D18" s="20"/>
-      <c r="E18" s="20"/>
-      <c r="F18" s="20"/>
-      <c r="G18" s="20"/>
-      <c r="H18" s="20"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="28" t="s">
+      <c r="B18" s="3"/>
+      <c r="C18" s="3"/>
+      <c r="D18" s="3"/>
+      <c r="E18" s="3"/>
+      <c r="F18" s="3"/>
+      <c r="G18" s="3"/>
+      <c r="H18" s="3"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B19" s="29" t="n">
+      <c r="B19" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="C19" s="29" t="n">
+      <c r="C19" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D19" s="29" t="n">
+      <c r="D19" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="E19" s="29" t="n">
+      <c r="E19" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="F19" s="29" t="n">
+      <c r="F19" s="22" t="n">
         <v>250</v>
       </c>
-      <c r="G19" s="29" t="n">
+      <c r="G19" s="22" t="n">
         <v>1000</v>
       </c>
-      <c r="H19" s="20"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="20" t="s">
+      <c r="H19" s="3"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
         <v>80</v>
       </c>
-      <c r="B20" s="30" t="n">
+      <c r="B20" s="23" t="n">
         <f aca="false">B$19*$B$10</f>
-        <v>1500</v>
-      </c>
-      <c r="C20" s="30" t="n">
+        <v>3000</v>
+      </c>
+      <c r="C20" s="23" t="n">
         <f aca="false">C$19*$B$10</f>
-        <v>3750</v>
-      </c>
-      <c r="D20" s="30" t="n">
+        <v>7500</v>
+      </c>
+      <c r="D20" s="23" t="n">
         <f aca="false">D$19*$B$10</f>
-        <v>7500</v>
-      </c>
-      <c r="E20" s="30" t="n">
+        <v>15000</v>
+      </c>
+      <c r="E20" s="23" t="n">
         <f aca="false">E$19*$B$10</f>
-        <v>15000</v>
-      </c>
-      <c r="F20" s="30" t="n">
+        <v>30000</v>
+      </c>
+      <c r="F20" s="23" t="n">
         <f aca="false">F$19*$B$10</f>
-        <v>37500</v>
-      </c>
-      <c r="G20" s="30" t="n">
+        <v>75000</v>
+      </c>
+      <c r="G20" s="23" t="n">
         <f aca="false">G$19*$B$10</f>
-        <v>150000</v>
-      </c>
-      <c r="H20" s="20"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="20" t="s">
+        <v>300000</v>
+      </c>
+      <c r="H20" s="3"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A21" s="3" t="s">
         <v>81</v>
       </c>
-      <c r="B21" s="30" t="n">
+      <c r="B21" s="23" t="n">
         <f aca="false">B20*$B$13</f>
-        <v>33.75</v>
-      </c>
-      <c r="C21" s="30" t="n">
+        <v>270</v>
+      </c>
+      <c r="C21" s="23" t="n">
         <f aca="false">C20*$B$13</f>
-        <v>84.375</v>
-      </c>
-      <c r="D21" s="30" t="n">
+        <v>675</v>
+      </c>
+      <c r="D21" s="23" t="n">
         <f aca="false">D20*$B$13</f>
-        <v>168.75</v>
-      </c>
-      <c r="E21" s="30" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E21" s="23" t="n">
         <f aca="false">E20*$B$13</f>
-        <v>337.5</v>
-      </c>
-      <c r="F21" s="30" t="n">
+        <v>2700</v>
+      </c>
+      <c r="F21" s="23" t="n">
         <f aca="false">F20*$B$13</f>
-        <v>843.75</v>
-      </c>
-      <c r="G21" s="30" t="n">
+        <v>6750</v>
+      </c>
+      <c r="G21" s="23" t="n">
         <f aca="false">G20*$B$13</f>
-        <v>3375</v>
-      </c>
-      <c r="H21" s="20"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="20" t="s">
+        <v>27000</v>
+      </c>
+      <c r="H21" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="B22" s="30" t="n">
+      <c r="B22" s="23" t="n">
         <f aca="false">B20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+B20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>11.625</v>
-      </c>
-      <c r="C22" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="C22" s="23" t="n">
         <f aca="false">C20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+C20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>29.0625</v>
-      </c>
-      <c r="D22" s="30" t="n">
+        <v>7.50000000000001</v>
+      </c>
+      <c r="D22" s="23" t="n">
         <f aca="false">D20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+D20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>58.125</v>
-      </c>
-      <c r="E22" s="30" t="n">
+        <v>15</v>
+      </c>
+      <c r="E22" s="23" t="n">
         <f aca="false">E20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+E20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>116.25</v>
-      </c>
-      <c r="F22" s="30" t="n">
+        <v>30</v>
+      </c>
+      <c r="F22" s="23" t="n">
         <f aca="false">F20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+F20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>290.625</v>
-      </c>
-      <c r="G22" s="30" t="n">
+        <v>75.0000000000001</v>
+      </c>
+      <c r="G22" s="23" t="n">
         <f aca="false">G20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+G20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>1162.5</v>
-      </c>
-      <c r="H22" s="20"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="20" t="s">
+        <v>300</v>
+      </c>
+      <c r="H22" s="3"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A23" s="3" t="s">
         <v>83</v>
       </c>
-      <c r="B23" s="30" t="n">
+      <c r="B23" s="23" t="n">
         <f aca="false">B$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>40.8333333333333</v>
-      </c>
-      <c r="C23" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="C23" s="23" t="n">
         <f aca="false">C$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>102.083333333333</v>
-      </c>
-      <c r="D23" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="23" t="n">
         <f aca="false">D$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>204.166666666667</v>
-      </c>
-      <c r="E23" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="23" t="n">
         <f aca="false">E$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>408.333333333333</v>
-      </c>
-      <c r="F23" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="23" t="n">
         <f aca="false">F$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>1020.83333333333</v>
-      </c>
-      <c r="G23" s="30" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="23" t="n">
         <f aca="false">G$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>4083.33333333333</v>
-      </c>
-      <c r="H23" s="20"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="H23" s="3"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A24" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B24" s="31" t="n">
+      <c r="B24" s="24" t="n">
         <f aca="false">SUM(B21:B23)</f>
-        <v>86.2083333333333</v>
-      </c>
-      <c r="C24" s="31" t="n">
+        <v>273</v>
+      </c>
+      <c r="C24" s="24" t="n">
         <f aca="false">SUM(C21:C23)</f>
-        <v>215.520833333333</v>
-      </c>
-      <c r="D24" s="31" t="n">
+        <v>682.5</v>
+      </c>
+      <c r="D24" s="24" t="n">
         <f aca="false">SUM(D21:D23)</f>
-        <v>431.041666666667</v>
-      </c>
-      <c r="E24" s="31" t="n">
+        <v>1365</v>
+      </c>
+      <c r="E24" s="24" t="n">
         <f aca="false">SUM(E21:E23)</f>
-        <v>862.083333333333</v>
-      </c>
-      <c r="F24" s="31" t="n">
+        <v>2730</v>
+      </c>
+      <c r="F24" s="24" t="n">
         <f aca="false">SUM(F21:F23)</f>
-        <v>2155.20833333333</v>
-      </c>
-      <c r="G24" s="31" t="n">
+        <v>6825</v>
+      </c>
+      <c r="G24" s="24" t="n">
         <f aca="false">SUM(G21:G23)</f>
-        <v>8620.83333333333</v>
-      </c>
-      <c r="H24" s="20"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="20" t="s">
+        <v>27300</v>
+      </c>
+      <c r="H24" s="3"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A25" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="30" t="n">
+      <c r="B25" s="23" t="n">
         <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),B$19*Supuestos!$B$43)</f>
-        <v>16.2</v>
-      </c>
-      <c r="C25" s="30" t="n">
+        <v>162</v>
+      </c>
+      <c r="C25" s="23" t="n">
         <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),C$19*Supuestos!$B$43)</f>
-        <v>16.2</v>
-      </c>
-      <c r="D25" s="30" t="n">
+        <v>405</v>
+      </c>
+      <c r="D25" s="23" t="n">
         <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),D$19*Supuestos!$B$43)</f>
-        <v>16.2</v>
-      </c>
-      <c r="E25" s="30" t="n">
+        <v>810</v>
+      </c>
+      <c r="E25" s="23" t="n">
         <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),E$19*Supuestos!$B$43)</f>
-        <v>16.2</v>
-      </c>
-      <c r="F25" s="30" t="n">
+        <v>1620</v>
+      </c>
+      <c r="F25" s="23" t="n">
         <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),F$19*Supuestos!$B$43)</f>
-        <v>16.2</v>
-      </c>
-      <c r="G25" s="30" t="n">
+        <v>4050</v>
+      </c>
+      <c r="G25" s="23" t="n">
         <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),G$19*Supuestos!$B$43)</f>
-        <v>16.2</v>
-      </c>
-      <c r="H25" s="20"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="20" t="s">
+        <v>16200</v>
+      </c>
+      <c r="H25" s="3"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A26" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B26" s="30" t="n">
+      <c r="B26" s="23" t="n">
         <f aca="false">IF(B$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>49</v>
       </c>
-      <c r="C26" s="30" t="n">
+      <c r="C26" s="23" t="n">
         <f aca="false">IF(C$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>49</v>
       </c>
-      <c r="D26" s="30" t="n">
+      <c r="D26" s="23" t="n">
         <f aca="false">IF(D$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="E26" s="30" t="n">
+      <c r="E26" s="23" t="n">
         <f aca="false">IF(E$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="F26" s="30" t="n">
+      <c r="F26" s="23" t="n">
         <f aca="false">IF(F$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="G26" s="30" t="n">
+      <c r="G26" s="23" t="n">
         <f aca="false">IF(G$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="H26" s="20"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="20" t="s">
+      <c r="H26" s="3"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A27" s="3" t="s">
         <v>87</v>
       </c>
-      <c r="B27" s="30" t="n">
+      <c r="B27" s="23" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="C27" s="30" t="n">
+      <c r="C27" s="23" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="D27" s="30" t="n">
+      <c r="D27" s="23" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="E27" s="30" t="n">
+      <c r="E27" s="23" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="F27" s="30" t="n">
+      <c r="F27" s="23" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="G27" s="30" t="n">
+      <c r="G27" s="23" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="H27" s="20"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="20" t="s">
+      <c r="H27" s="3"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B28" s="31" t="n">
+      <c r="B28" s="24" t="n">
         <f aca="false">SUM(B25:B27)</f>
-        <v>325.2</v>
-      </c>
-      <c r="C28" s="31" t="n">
+        <v>471</v>
+      </c>
+      <c r="C28" s="24" t="n">
         <f aca="false">SUM(C25:C27)</f>
-        <v>325.2</v>
-      </c>
-      <c r="D28" s="31" t="n">
+        <v>714</v>
+      </c>
+      <c r="D28" s="24" t="n">
         <f aca="false">SUM(D25:D27)</f>
-        <v>525.2</v>
-      </c>
-      <c r="E28" s="31" t="n">
+        <v>1319</v>
+      </c>
+      <c r="E28" s="24" t="n">
         <f aca="false">SUM(E25:E27)</f>
-        <v>525.2</v>
-      </c>
-      <c r="F28" s="31" t="n">
+        <v>2129</v>
+      </c>
+      <c r="F28" s="24" t="n">
         <f aca="false">SUM(F25:F27)</f>
-        <v>525.2</v>
-      </c>
-      <c r="G28" s="31" t="n">
+        <v>4559</v>
+      </c>
+      <c r="G28" s="24" t="n">
         <f aca="false">SUM(G25:G27)</f>
-        <v>525.2</v>
-      </c>
-      <c r="H28" s="20"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="20" t="s">
+        <v>16709</v>
+      </c>
+      <c r="H28" s="3"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A29" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B29" s="31" t="n">
+      <c r="B29" s="24" t="n">
         <f aca="false">B24-B28</f>
-        <v>-238.991666666667</v>
-      </c>
-      <c r="C29" s="31" t="n">
+        <v>-198</v>
+      </c>
+      <c r="C29" s="24" t="n">
         <f aca="false">C24-C28</f>
-        <v>-109.679166666667</v>
-      </c>
-      <c r="D29" s="31" t="n">
+        <v>-31.4999999999999</v>
+      </c>
+      <c r="D29" s="24" t="n">
         <f aca="false">D24-D28</f>
-        <v>-94.1583333333334</v>
-      </c>
-      <c r="E29" s="31" t="n">
+        <v>46.0000000000002</v>
+      </c>
+      <c r="E29" s="24" t="n">
         <f aca="false">E24-E28</f>
-        <v>336.883333333333</v>
-      </c>
-      <c r="F29" s="31" t="n">
+        <v>601.000000000001</v>
+      </c>
+      <c r="F29" s="24" t="n">
         <f aca="false">F24-F28</f>
-        <v>1630.00833333333</v>
-      </c>
-      <c r="G29" s="31" t="n">
+        <v>2266</v>
+      </c>
+      <c r="G29" s="24" t="n">
         <f aca="false">G24-G28</f>
-        <v>8095.63333333333</v>
-      </c>
-      <c r="H29" s="20"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="20" t="s">
+        <v>10591</v>
+      </c>
+      <c r="H29" s="3"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A30" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="B30" s="30" t="n">
+      <c r="B30" s="23" t="n">
         <f aca="false">B29*12</f>
-        <v>-2867.9</v>
-      </c>
-      <c r="C30" s="30" t="n">
+        <v>-2376</v>
+      </c>
+      <c r="C30" s="23" t="n">
         <f aca="false">C29*12</f>
-        <v>-1316.15</v>
-      </c>
-      <c r="D30" s="30" t="n">
+        <v>-377.999999999999</v>
+      </c>
+      <c r="D30" s="23" t="n">
         <f aca="false">D29*12</f>
-        <v>-1129.9</v>
-      </c>
-      <c r="E30" s="30" t="n">
+        <v>552.000000000003</v>
+      </c>
+      <c r="E30" s="23" t="n">
         <f aca="false">E29*12</f>
-        <v>4042.6</v>
-      </c>
-      <c r="F30" s="30" t="n">
+        <v>7212.00000000001</v>
+      </c>
+      <c r="F30" s="23" t="n">
         <f aca="false">F29*12</f>
-        <v>19560.1</v>
-      </c>
-      <c r="G30" s="30" t="n">
+        <v>27192</v>
+      </c>
+      <c r="G30" s="23" t="n">
         <f aca="false">G29*12</f>
-        <v>97147.6</v>
-      </c>
-      <c r="H30" s="20"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="20" t="s">
+        <v>127092</v>
+      </c>
+      <c r="H30" s="3"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A31" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="30" t="n">
+      <c r="B31" s="23" t="n">
         <f aca="false">IF(B$19=0,0,B24/B$19)</f>
-        <v>8.62083333333333</v>
-      </c>
-      <c r="C31" s="30" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="C31" s="23" t="n">
         <f aca="false">IF(C$19=0,0,C24/C$19)</f>
-        <v>8.62083333333333</v>
-      </c>
-      <c r="D31" s="30" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="D31" s="23" t="n">
         <f aca="false">IF(D$19=0,0,D24/D$19)</f>
-        <v>8.62083333333333</v>
-      </c>
-      <c r="E31" s="30" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="E31" s="23" t="n">
         <f aca="false">IF(E$19=0,0,E24/E$19)</f>
-        <v>8.62083333333333</v>
-      </c>
-      <c r="F31" s="30" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="F31" s="23" t="n">
         <f aca="false">IF(F$19=0,0,F24/F$19)</f>
-        <v>8.62083333333333</v>
-      </c>
-      <c r="G31" s="30" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="G31" s="23" t="n">
         <f aca="false">IF(G$19=0,0,G24/G$19)</f>
-        <v>8.62083333333333</v>
-      </c>
-      <c r="H31" s="20"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="20" t="s">
+        <v>27.3</v>
+      </c>
+      <c r="H31" s="3"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A32" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="B32" s="30" t="n">
+      <c r="B32" s="23" t="n">
         <f aca="false">B21+B23</f>
-        <v>74.5833333333333</v>
-      </c>
-      <c r="C32" s="30" t="n">
+        <v>270</v>
+      </c>
+      <c r="C32" s="23" t="n">
         <f aca="false">C21+C23</f>
-        <v>186.458333333333</v>
-      </c>
-      <c r="D32" s="30" t="n">
+        <v>675</v>
+      </c>
+      <c r="D32" s="23" t="n">
         <f aca="false">D21+D23</f>
-        <v>372.916666666667</v>
-      </c>
-      <c r="E32" s="30" t="n">
+        <v>1350</v>
+      </c>
+      <c r="E32" s="23" t="n">
         <f aca="false">E21+E23</f>
-        <v>745.833333333333</v>
-      </c>
-      <c r="F32" s="30" t="n">
+        <v>2700</v>
+      </c>
+      <c r="F32" s="23" t="n">
         <f aca="false">F21+F23</f>
-        <v>1864.58333333333</v>
-      </c>
-      <c r="G32" s="30" t="n">
+        <v>6750</v>
+      </c>
+      <c r="G32" s="23" t="n">
         <f aca="false">G21+G23</f>
-        <v>7458.33333333333</v>
-      </c>
-      <c r="H32" s="20"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="20"/>
-      <c r="B33" s="20"/>
-      <c r="C33" s="20"/>
-      <c r="D33" s="20"/>
-      <c r="E33" s="20"/>
-      <c r="F33" s="20"/>
-      <c r="G33" s="20"/>
-      <c r="H33" s="20"/>
+        <v>27000</v>
+      </c>
+      <c r="H32" s="3"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A33" s="3"/>
+      <c r="B33" s="3"/>
+      <c r="C33" s="3"/>
+      <c r="D33" s="3"/>
+      <c r="E33" s="3"/>
+      <c r="F33" s="3"/>
+      <c r="G33" s="3"/>
+      <c r="H33" s="3"/>
     </row>
     <row r="34" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="32" t="s">
+      <c r="A34" s="25" t="s">
         <v>93</v>
       </c>
-      <c r="B34" s="32"/>
-      <c r="C34" s="32"/>
-      <c r="D34" s="32"/>
-      <c r="E34" s="32"/>
-      <c r="F34" s="32"/>
-      <c r="G34" s="32"/>
-      <c r="H34" s="32"/>
+      <c r="B34" s="25"/>
+      <c r="C34" s="25"/>
+      <c r="D34" s="25"/>
+      <c r="E34" s="25"/>
+      <c r="F34" s="25"/>
+      <c r="G34" s="25"/>
+      <c r="H34" s="25"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2254,22 +2205,22 @@
       <c r="A4" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="33" t="n">
+      <c r="B4" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="C4" s="33" t="n">
+      <c r="C4" s="22" t="n">
         <v>25</v>
       </c>
-      <c r="D4" s="33" t="n">
+      <c r="D4" s="22" t="n">
         <v>50</v>
       </c>
-      <c r="E4" s="33" t="n">
+      <c r="E4" s="22" t="n">
         <v>100</v>
       </c>
-      <c r="F4" s="33" t="n">
+      <c r="F4" s="22" t="n">
         <v>250</v>
       </c>
-      <c r="G4" s="33" t="n">
+      <c r="G4" s="22" t="n">
         <v>1000</v>
       </c>
     </row>
@@ -2277,27 +2228,27 @@
       <c r="A5" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B5" s="34" t="n">
+      <c r="B5" s="26" t="n">
         <f aca="false">B$4*Supuestos!$B$34</f>
         <v>10000</v>
       </c>
-      <c r="C5" s="34" t="n">
+      <c r="C5" s="26" t="n">
         <f aca="false">C$4*Supuestos!$B$34</f>
         <v>25000</v>
       </c>
-      <c r="D5" s="34" t="n">
+      <c r="D5" s="26" t="n">
         <f aca="false">D$4*Supuestos!$B$34</f>
         <v>50000</v>
       </c>
-      <c r="E5" s="34" t="n">
+      <c r="E5" s="26" t="n">
         <f aca="false">E$4*Supuestos!$B$34</f>
         <v>100000</v>
       </c>
-      <c r="F5" s="34" t="n">
+      <c r="F5" s="26" t="n">
         <f aca="false">F$4*Supuestos!$B$34</f>
         <v>250000</v>
       </c>
-      <c r="G5" s="34" t="n">
+      <c r="G5" s="26" t="n">
         <f aca="false">G$4*Supuestos!$B$34</f>
         <v>1000000</v>
       </c>
@@ -2306,27 +2257,27 @@
       <c r="A6" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B6" s="34" t="n">
+      <c r="B6" s="26" t="n">
         <f aca="false">B5*Supuestos!$B$35</f>
         <v>5000</v>
       </c>
-      <c r="C6" s="34" t="n">
+      <c r="C6" s="26" t="n">
         <f aca="false">C5*Supuestos!$B$35</f>
         <v>12500</v>
       </c>
-      <c r="D6" s="34" t="n">
+      <c r="D6" s="26" t="n">
         <f aca="false">D5*Supuestos!$B$35</f>
         <v>25000</v>
       </c>
-      <c r="E6" s="34" t="n">
+      <c r="E6" s="26" t="n">
         <f aca="false">E5*Supuestos!$B$35</f>
         <v>50000</v>
       </c>
-      <c r="F6" s="34" t="n">
+      <c r="F6" s="26" t="n">
         <f aca="false">F5*Supuestos!$B$35</f>
         <v>125000</v>
       </c>
-      <c r="G6" s="34" t="n">
+      <c r="G6" s="26" t="n">
         <f aca="false">G5*Supuestos!$B$35</f>
         <v>500000</v>
       </c>
@@ -2335,27 +2286,27 @@
       <c r="A7" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B7" s="34" t="n">
+      <c r="B7" s="26" t="n">
         <f aca="false">B5-B6</f>
         <v>5000</v>
       </c>
-      <c r="C7" s="34" t="n">
+      <c r="C7" s="26" t="n">
         <f aca="false">C5-C6</f>
         <v>12500</v>
       </c>
-      <c r="D7" s="34" t="n">
+      <c r="D7" s="26" t="n">
         <f aca="false">D5-D6</f>
         <v>25000</v>
       </c>
-      <c r="E7" s="34" t="n">
+      <c r="E7" s="26" t="n">
         <f aca="false">E5-E6</f>
         <v>50000</v>
       </c>
-      <c r="F7" s="34" t="n">
+      <c r="F7" s="26" t="n">
         <f aca="false">F5-F6</f>
         <v>125000</v>
       </c>
-      <c r="G7" s="34" t="n">
+      <c r="G7" s="26" t="n">
         <f aca="false">G5-G6</f>
         <v>500000</v>
       </c>
@@ -2364,27 +2315,27 @@
       <c r="A8" s="3" t="s">
         <v>99</v>
       </c>
-      <c r="B8" s="35" t="n">
+      <c r="B8" s="27" t="n">
         <f aca="false">B$4*Supuestos!$B$39</f>
         <v>1800</v>
       </c>
-      <c r="C8" s="35" t="n">
+      <c r="C8" s="27" t="n">
         <f aca="false">C$4*Supuestos!$B$39</f>
         <v>4500</v>
       </c>
-      <c r="D8" s="35" t="n">
+      <c r="D8" s="27" t="n">
         <f aca="false">D$4*Supuestos!$B$39</f>
         <v>9000</v>
       </c>
-      <c r="E8" s="35" t="n">
+      <c r="E8" s="27" t="n">
         <f aca="false">E$4*Supuestos!$B$39</f>
         <v>18000</v>
       </c>
-      <c r="F8" s="35" t="n">
+      <c r="F8" s="27" t="n">
         <f aca="false">F$4*Supuestos!$B$39</f>
         <v>45000</v>
       </c>
-      <c r="G8" s="35" t="n">
+      <c r="G8" s="27" t="n">
         <f aca="false">G$4*Supuestos!$B$39</f>
         <v>180000</v>
       </c>
@@ -2413,27 +2364,27 @@
       <c r="A11" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="B11" s="34" t="n">
+      <c r="B11" s="26" t="n">
         <f aca="false">B6*Supuestos!$B$41</f>
         <v>900</v>
       </c>
-      <c r="C11" s="34" t="n">
+      <c r="C11" s="26" t="n">
         <f aca="false">C6*Supuestos!$B$41</f>
         <v>2250</v>
       </c>
-      <c r="D11" s="34" t="n">
+      <c r="D11" s="26" t="n">
         <f aca="false">D6*Supuestos!$B$41</f>
         <v>4500</v>
       </c>
-      <c r="E11" s="34" t="n">
+      <c r="E11" s="26" t="n">
         <f aca="false">E6*Supuestos!$B$41</f>
         <v>9000</v>
       </c>
-      <c r="F11" s="34" t="n">
+      <c r="F11" s="26" t="n">
         <f aca="false">F6*Supuestos!$B$41</f>
         <v>22500</v>
       </c>
-      <c r="G11" s="34" t="n">
+      <c r="G11" s="26" t="n">
         <f aca="false">G6*Supuestos!$B$41</f>
         <v>90000</v>
       </c>
@@ -2442,27 +2393,27 @@
       <c r="A12" s="3" t="s">
         <v>102</v>
       </c>
-      <c r="B12" s="34" t="n">
+      <c r="B12" s="26" t="n">
         <f aca="false">B7*Supuestos!$B$42</f>
         <v>1800</v>
       </c>
-      <c r="C12" s="34" t="n">
+      <c r="C12" s="26" t="n">
         <f aca="false">C7*Supuestos!$B$42</f>
         <v>4500</v>
       </c>
-      <c r="D12" s="34" t="n">
+      <c r="D12" s="26" t="n">
         <f aca="false">D7*Supuestos!$B$42</f>
         <v>9000</v>
       </c>
-      <c r="E12" s="34" t="n">
+      <c r="E12" s="26" t="n">
         <f aca="false">E7*Supuestos!$B$42</f>
         <v>18000</v>
       </c>
-      <c r="F12" s="34" t="n">
+      <c r="F12" s="26" t="n">
         <f aca="false">F7*Supuestos!$B$42</f>
         <v>45000</v>
       </c>
-      <c r="G12" s="34" t="n">
+      <c r="G12" s="26" t="n">
         <f aca="false">G7*Supuestos!$B$42</f>
         <v>180000</v>
       </c>
@@ -2471,27 +2422,27 @@
       <c r="A13" s="3" t="s">
         <v>103</v>
       </c>
-      <c r="B13" s="34" t="n">
+      <c r="B13" s="26" t="n">
         <f aca="false">B7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
-      <c r="C13" s="34" t="n">
+      <c r="C13" s="26" t="n">
         <f aca="false">C7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
-      <c r="D13" s="34" t="n">
+      <c r="D13" s="26" t="n">
         <f aca="false">D7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
-      <c r="E13" s="34" t="n">
+      <c r="E13" s="26" t="n">
         <f aca="false">E7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
-      <c r="F13" s="34" t="n">
+      <c r="F13" s="26" t="n">
         <f aca="false">F7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
-      <c r="G13" s="34" t="n">
+      <c r="G13" s="26" t="n">
         <f aca="false">G7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
@@ -2500,27 +2451,27 @@
       <c r="A14" s="3" t="s">
         <v>104</v>
       </c>
-      <c r="B14" s="34" t="n">
+      <c r="B14" s="26" t="n">
         <f aca="false">B6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="C14" s="34" t="n">
+      <c r="C14" s="26" t="n">
         <f aca="false">C6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="D14" s="34" t="n">
+      <c r="D14" s="26" t="n">
         <f aca="false">D6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="E14" s="34" t="n">
+      <c r="E14" s="26" t="n">
         <f aca="false">E6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="F14" s="34" t="n">
+      <c r="F14" s="26" t="n">
         <f aca="false">F6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="G14" s="34" t="n">
+      <c r="G14" s="26" t="n">
         <f aca="false">G6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
@@ -2529,27 +2480,27 @@
       <c r="A15" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B15" s="34" t="n">
+      <c r="B15" s="26" t="n">
         <f aca="false">SUM(B11:B14)</f>
         <v>2700</v>
       </c>
-      <c r="C15" s="34" t="n">
+      <c r="C15" s="26" t="n">
         <f aca="false">SUM(C11:C14)</f>
         <v>6750</v>
       </c>
-      <c r="D15" s="34" t="n">
+      <c r="D15" s="26" t="n">
         <f aca="false">SUM(D11:D14)</f>
         <v>13500</v>
       </c>
-      <c r="E15" s="34" t="n">
+      <c r="E15" s="26" t="n">
         <f aca="false">SUM(E11:E14)</f>
         <v>27000</v>
       </c>
-      <c r="F15" s="34" t="n">
+      <c r="F15" s="26" t="n">
         <f aca="false">SUM(F11:F14)</f>
         <v>67500</v>
       </c>
-      <c r="G15" s="34" t="n">
+      <c r="G15" s="26" t="n">
         <f aca="false">SUM(G11:G14)</f>
         <v>270000</v>
       </c>
@@ -2578,27 +2529,27 @@
       <c r="A18" s="3" t="s">
         <v>106</v>
       </c>
-      <c r="B18" s="34" t="n">
+      <c r="B18" s="26" t="n">
         <f aca="false">B$4*Supuestos!$B$43</f>
         <v>162</v>
       </c>
-      <c r="C18" s="34" t="n">
+      <c r="C18" s="26" t="n">
         <f aca="false">C$4*Supuestos!$B$43</f>
         <v>405</v>
       </c>
-      <c r="D18" s="34" t="n">
+      <c r="D18" s="26" t="n">
         <f aca="false">D$4*Supuestos!$B$43</f>
         <v>810</v>
       </c>
-      <c r="E18" s="34" t="n">
+      <c r="E18" s="26" t="n">
         <f aca="false">E$4*Supuestos!$B$43</f>
         <v>1620</v>
       </c>
-      <c r="F18" s="34" t="n">
+      <c r="F18" s="26" t="n">
         <f aca="false">F$4*Supuestos!$B$43</f>
         <v>4050</v>
       </c>
-      <c r="G18" s="34" t="n">
+      <c r="G18" s="26" t="n">
         <f aca="false">G$4*Supuestos!$B$43</f>
         <v>16200</v>
       </c>
@@ -2607,27 +2558,27 @@
       <c r="A19" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="B19" s="34" t="n">
+      <c r="B19" s="26" t="n">
         <f aca="false">IF(B$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>49</v>
       </c>
-      <c r="C19" s="34" t="n">
+      <c r="C19" s="26" t="n">
         <f aca="false">IF(C$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>49</v>
       </c>
-      <c r="D19" s="34" t="n">
+      <c r="D19" s="26" t="n">
         <f aca="false">IF(D$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="E19" s="34" t="n">
+      <c r="E19" s="26" t="n">
         <f aca="false">IF(E$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="F19" s="34" t="n">
+      <c r="F19" s="26" t="n">
         <f aca="false">IF(F$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="G19" s="34" t="n">
+      <c r="G19" s="26" t="n">
         <f aca="false">IF(G$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
@@ -2636,27 +2587,27 @@
       <c r="A20" s="3" t="s">
         <v>107</v>
       </c>
-      <c r="B20" s="34" t="n">
+      <c r="B20" s="26" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="C20" s="34" t="n">
+      <c r="C20" s="26" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="D20" s="34" t="n">
+      <c r="D20" s="26" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="E20" s="34" t="n">
+      <c r="E20" s="26" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="F20" s="34" t="n">
+      <c r="F20" s="26" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
-      <c r="G20" s="34" t="n">
+      <c r="G20" s="26" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
         <v>260</v>
       </c>
@@ -2665,27 +2616,27 @@
       <c r="A21" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B21" s="34" t="n">
+      <c r="B21" s="26" t="n">
         <f aca="false">SUM(B18:B20)</f>
         <v>471</v>
       </c>
-      <c r="C21" s="34" t="n">
+      <c r="C21" s="26" t="n">
         <f aca="false">SUM(C18:C20)</f>
         <v>714</v>
       </c>
-      <c r="D21" s="34" t="n">
+      <c r="D21" s="26" t="n">
         <f aca="false">SUM(D18:D20)</f>
         <v>1319</v>
       </c>
-      <c r="E21" s="34" t="n">
+      <c r="E21" s="26" t="n">
         <f aca="false">SUM(E18:E20)</f>
         <v>2129</v>
       </c>
-      <c r="F21" s="34" t="n">
+      <c r="F21" s="26" t="n">
         <f aca="false">SUM(F18:F20)</f>
         <v>4559</v>
       </c>
-      <c r="G21" s="34" t="n">
+      <c r="G21" s="26" t="n">
         <f aca="false">SUM(G18:G20)</f>
         <v>16709</v>
       </c>
@@ -2703,27 +2654,27 @@
       <c r="A23" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B23" s="36" t="n">
+      <c r="B23" s="24" t="n">
         <f aca="false">B15-B21</f>
         <v>2229</v>
       </c>
-      <c r="C23" s="36" t="n">
+      <c r="C23" s="24" t="n">
         <f aca="false">C15-C21</f>
         <v>6036</v>
       </c>
-      <c r="D23" s="36" t="n">
+      <c r="D23" s="24" t="n">
         <f aca="false">D15-D21</f>
         <v>12181</v>
       </c>
-      <c r="E23" s="36" t="n">
+      <c r="E23" s="24" t="n">
         <f aca="false">E15-E21</f>
         <v>24871</v>
       </c>
-      <c r="F23" s="36" t="n">
+      <c r="F23" s="24" t="n">
         <f aca="false">F15-F21</f>
         <v>62941</v>
       </c>
-      <c r="G23" s="36" t="n">
+      <c r="G23" s="24" t="n">
         <f aca="false">G15-G21</f>
         <v>253291</v>
       </c>
@@ -2761,27 +2712,27 @@
       <c r="A25" s="3" t="s">
         <v>91</v>
       </c>
-      <c r="B25" s="34" t="n">
+      <c r="B25" s="26" t="n">
         <f aca="false">IF(B$4=0,0,B15/B$4)</f>
         <v>270</v>
       </c>
-      <c r="C25" s="34" t="n">
+      <c r="C25" s="26" t="n">
         <f aca="false">IF(C$4=0,0,C15/C$4)</f>
         <v>270</v>
       </c>
-      <c r="D25" s="34" t="n">
+      <c r="D25" s="26" t="n">
         <f aca="false">IF(D$4=0,0,D15/D$4)</f>
         <v>270</v>
       </c>
-      <c r="E25" s="34" t="n">
+      <c r="E25" s="26" t="n">
         <f aca="false">IF(E$4=0,0,E15/E$4)</f>
         <v>270</v>
       </c>
-      <c r="F25" s="34" t="n">
+      <c r="F25" s="26" t="n">
         <f aca="false">IF(F$4=0,0,F15/F$4)</f>
         <v>270</v>
       </c>
-      <c r="G25" s="34" t="n">
+      <c r="G25" s="26" t="n">
         <f aca="false">IF(G$4=0,0,G15/G$4)</f>
         <v>270</v>
       </c>
@@ -2897,27 +2848,27 @@
       <c r="A31" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B31" s="37" t="n">
+      <c r="B31" s="20" t="n">
         <f aca="false">B28+B29+B30</f>
         <v>-0.26</v>
       </c>
-      <c r="C31" s="37" t="n">
+      <c r="C31" s="20" t="n">
         <f aca="false">C28+C29+C30</f>
         <v>-0.26</v>
       </c>
-      <c r="D31" s="37" t="n">
+      <c r="D31" s="20" t="n">
         <f aca="false">D28+D29+D30</f>
         <v>-0.26</v>
       </c>
-      <c r="E31" s="37" t="n">
+      <c r="E31" s="20" t="n">
         <f aca="false">E28+E29+E30</f>
         <v>-0.26</v>
       </c>
-      <c r="F31" s="37" t="n">
+      <c r="F31" s="20" t="n">
         <f aca="false">F28+F29+F30</f>
         <v>-0.26</v>
       </c>
-      <c r="G31" s="37" t="n">
+      <c r="G31" s="20" t="n">
         <f aca="false">G28+G29+G30</f>
         <v>-0.26</v>
       </c>
@@ -2926,27 +2877,27 @@
       <c r="A32" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B32" s="37" t="n">
+      <c r="B32" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="C32" s="37" t="n">
+      <c r="C32" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="D32" s="37" t="n">
+      <c r="D32" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="E32" s="37" t="n">
+      <c r="E32" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="F32" s="37" t="n">
+      <c r="F32" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="G32" s="37" t="n">
+      <c r="G32" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
@@ -3061,27 +3012,27 @@
       <c r="A5" s="8" t="n">
         <v>-0.1</v>
       </c>
-      <c r="B5" s="38" t="n">
+      <c r="B5" s="21" t="n">
         <f aca="false">$A5-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.22</v>
       </c>
-      <c r="C5" s="38" t="n">
+      <c r="C5" s="21" t="n">
         <f aca="false">$A5-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.34</v>
       </c>
-      <c r="D5" s="38" t="n">
+      <c r="D5" s="21" t="n">
         <f aca="false">$A5-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.46</v>
       </c>
-      <c r="E5" s="38" t="n">
+      <c r="E5" s="21" t="n">
         <f aca="false">$A5-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.58</v>
       </c>
-      <c r="F5" s="38" t="n">
+      <c r="F5" s="21" t="n">
         <f aca="false">$A5-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.7</v>
       </c>
-      <c r="G5" s="38" t="n">
+      <c r="G5" s="21" t="n">
         <f aca="false">$A5-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-1</v>
       </c>
@@ -3090,27 +3041,27 @@
       <c r="A6" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="B6" s="38" t="n">
+      <c r="B6" s="21" t="n">
         <f aca="false">$A6-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.12</v>
       </c>
-      <c r="C6" s="38" t="n">
+      <c r="C6" s="21" t="n">
         <f aca="false">$A6-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.24</v>
       </c>
-      <c r="D6" s="38" t="n">
+      <c r="D6" s="21" t="n">
         <f aca="false">$A6-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.36</v>
       </c>
-      <c r="E6" s="38" t="n">
+      <c r="E6" s="21" t="n">
         <f aca="false">$A6-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.48</v>
       </c>
-      <c r="F6" s="38" t="n">
+      <c r="F6" s="21" t="n">
         <f aca="false">$A6-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.6</v>
       </c>
-      <c r="G6" s="38" t="n">
+      <c r="G6" s="21" t="n">
         <f aca="false">$A6-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.9</v>
       </c>
@@ -3119,27 +3070,27 @@
       <c r="A7" s="8" t="n">
         <v>0.05</v>
       </c>
-      <c r="B7" s="38" t="n">
+      <c r="B7" s="21" t="n">
         <f aca="false">$A7-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.07</v>
       </c>
-      <c r="C7" s="38" t="n">
+      <c r="C7" s="21" t="n">
         <f aca="false">$A7-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.19</v>
       </c>
-      <c r="D7" s="38" t="n">
+      <c r="D7" s="21" t="n">
         <f aca="false">$A7-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.31</v>
       </c>
-      <c r="E7" s="38" t="n">
+      <c r="E7" s="21" t="n">
         <f aca="false">$A7-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.43</v>
       </c>
-      <c r="F7" s="38" t="n">
+      <c r="F7" s="21" t="n">
         <f aca="false">$A7-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.55</v>
       </c>
-      <c r="G7" s="38" t="n">
+      <c r="G7" s="21" t="n">
         <f aca="false">$A7-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.85</v>
       </c>
@@ -3148,27 +3099,27 @@
       <c r="A8" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="B8" s="38" t="n">
+      <c r="B8" s="21" t="n">
         <f aca="false">$A8-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.02</v>
       </c>
-      <c r="C8" s="38" t="n">
+      <c r="C8" s="21" t="n">
         <f aca="false">$A8-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.14</v>
       </c>
-      <c r="D8" s="38" t="n">
+      <c r="D8" s="21" t="n">
         <f aca="false">$A8-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.26</v>
       </c>
-      <c r="E8" s="38" t="n">
+      <c r="E8" s="21" t="n">
         <f aca="false">$A8-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.38</v>
       </c>
-      <c r="F8" s="38" t="n">
+      <c r="F8" s="21" t="n">
         <f aca="false">$A8-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.5</v>
       </c>
-      <c r="G8" s="38" t="n">
+      <c r="G8" s="21" t="n">
         <f aca="false">$A8-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.8</v>
       </c>
@@ -3177,27 +3128,27 @@
       <c r="A9" s="8" t="n">
         <v>0.2</v>
       </c>
-      <c r="B9" s="38" t="n">
+      <c r="B9" s="21" t="n">
         <f aca="false">$A9-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.072</v>
       </c>
-      <c r="C9" s="38" t="n">
+      <c r="C9" s="21" t="n">
         <f aca="false">$A9-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.04</v>
       </c>
-      <c r="D9" s="38" t="n">
+      <c r="D9" s="21" t="n">
         <f aca="false">$A9-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.16</v>
       </c>
-      <c r="E9" s="38" t="n">
+      <c r="E9" s="21" t="n">
         <f aca="false">$A9-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.28</v>
       </c>
-      <c r="F9" s="38" t="n">
+      <c r="F9" s="21" t="n">
         <f aca="false">$A9-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.4</v>
       </c>
-      <c r="G9" s="38" t="n">
+      <c r="G9" s="21" t="n">
         <f aca="false">$A9-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.7</v>
       </c>
@@ -3206,27 +3157,27 @@
       <c r="A10" s="8" t="n">
         <v>0.3</v>
       </c>
-      <c r="B10" s="38" t="n">
+      <c r="B10" s="21" t="n">
         <f aca="false">$A10-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.162</v>
       </c>
-      <c r="C10" s="38" t="n">
+      <c r="C10" s="21" t="n">
         <f aca="false">$A10-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.054</v>
       </c>
-      <c r="D10" s="38" t="n">
+      <c r="D10" s="21" t="n">
         <f aca="false">$A10-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.06</v>
       </c>
-      <c r="E10" s="38" t="n">
+      <c r="E10" s="21" t="n">
         <f aca="false">$A10-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.18</v>
       </c>
-      <c r="F10" s="38" t="n">
+      <c r="F10" s="21" t="n">
         <f aca="false">$A10-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.3</v>
       </c>
-      <c r="G10" s="38" t="n">
+      <c r="G10" s="21" t="n">
         <f aca="false">$A10-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.6</v>
       </c>
@@ -3235,27 +3186,27 @@
       <c r="A11" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="B11" s="38" t="n">
+      <c r="B11" s="21" t="n">
         <f aca="false">$A11-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.342</v>
       </c>
-      <c r="C11" s="38" t="n">
+      <c r="C11" s="21" t="n">
         <f aca="false">$A11-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.234</v>
       </c>
-      <c r="D11" s="38" t="n">
+      <c r="D11" s="21" t="n">
         <f aca="false">$A11-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.126</v>
       </c>
-      <c r="E11" s="38" t="n">
+      <c r="E11" s="21" t="n">
         <f aca="false">$A11-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.018</v>
       </c>
-      <c r="F11" s="38" t="n">
+      <c r="F11" s="21" t="n">
         <f aca="false">$A11-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.1</v>
       </c>
-      <c r="G11" s="38" t="n">
+      <c r="G11" s="21" t="n">
         <f aca="false">$A11-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.4</v>
       </c>
@@ -3282,237 +3233,237 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3"/>
-      <c r="B14" s="39" t="n">
+      <c r="B14" s="28" t="n">
         <f aca="false">B$4</f>
         <v>0.2</v>
       </c>
-      <c r="C14" s="39" t="n">
+      <c r="C14" s="28" t="n">
         <f aca="false">C$4</f>
         <v>0.4</v>
       </c>
-      <c r="D14" s="39" t="n">
+      <c r="D14" s="28" t="n">
         <f aca="false">D$4</f>
         <v>0.6</v>
       </c>
-      <c r="E14" s="39" t="n">
+      <c r="E14" s="28" t="n">
         <f aca="false">E$4</f>
         <v>0.8</v>
       </c>
-      <c r="F14" s="39" t="n">
+      <c r="F14" s="28" t="n">
         <f aca="false">F$4</f>
         <v>1</v>
       </c>
-      <c r="G14" s="39" t="n">
+      <c r="G14" s="28" t="n">
         <f aca="false">G$4</f>
         <v>1.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="38" t="n">
+      <c r="A15" s="21" t="n">
         <f aca="false">$A5</f>
         <v>-0.1</v>
       </c>
-      <c r="B15" s="38" t="n">
+      <c r="B15" s="21" t="n">
         <f aca="false">$A15-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.16</v>
       </c>
-      <c r="C15" s="38" t="n">
+      <c r="C15" s="21" t="n">
         <f aca="false">$A15-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.22</v>
       </c>
-      <c r="D15" s="38" t="n">
+      <c r="D15" s="21" t="n">
         <f aca="false">$A15-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.28</v>
       </c>
-      <c r="E15" s="38" t="n">
+      <c r="E15" s="21" t="n">
         <f aca="false">$A15-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.34</v>
       </c>
-      <c r="F15" s="38" t="n">
+      <c r="F15" s="21" t="n">
         <f aca="false">$A15-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.4</v>
       </c>
-      <c r="G15" s="38" t="n">
+      <c r="G15" s="21" t="n">
         <f aca="false">$A15-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="38" t="n">
+      <c r="A16" s="21" t="n">
         <f aca="false">$A6</f>
         <v>0</v>
       </c>
-      <c r="B16" s="38" t="n">
+      <c r="B16" s="21" t="n">
         <f aca="false">$A16-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.06</v>
       </c>
-      <c r="C16" s="38" t="n">
+      <c r="C16" s="21" t="n">
         <f aca="false">$A16-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.12</v>
       </c>
-      <c r="D16" s="38" t="n">
+      <c r="D16" s="21" t="n">
         <f aca="false">$A16-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.18</v>
       </c>
-      <c r="E16" s="38" t="n">
+      <c r="E16" s="21" t="n">
         <f aca="false">$A16-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.24</v>
       </c>
-      <c r="F16" s="38" t="n">
+      <c r="F16" s="21" t="n">
         <f aca="false">$A16-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.3</v>
       </c>
-      <c r="G16" s="38" t="n">
+      <c r="G16" s="21" t="n">
         <f aca="false">$A16-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="38" t="n">
+      <c r="A17" s="21" t="n">
         <f aca="false">$A7</f>
         <v>0.05</v>
       </c>
-      <c r="B17" s="38" t="n">
+      <c r="B17" s="21" t="n">
         <f aca="false">$A17-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.01</v>
       </c>
-      <c r="C17" s="38" t="n">
+      <c r="C17" s="21" t="n">
         <f aca="false">$A17-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.07</v>
       </c>
-      <c r="D17" s="38" t="n">
+      <c r="D17" s="21" t="n">
         <f aca="false">$A17-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.13</v>
       </c>
-      <c r="E17" s="38" t="n">
+      <c r="E17" s="21" t="n">
         <f aca="false">$A17-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.19</v>
       </c>
-      <c r="F17" s="38" t="n">
+      <c r="F17" s="21" t="n">
         <f aca="false">$A17-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.25</v>
       </c>
-      <c r="G17" s="38" t="n">
+      <c r="G17" s="21" t="n">
         <f aca="false">$A17-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.4</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="38" t="n">
+      <c r="A18" s="21" t="n">
         <f aca="false">$A8</f>
         <v>0.1</v>
       </c>
-      <c r="B18" s="38" t="n">
+      <c r="B18" s="21" t="n">
         <f aca="false">$A18-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.04</v>
       </c>
-      <c r="C18" s="38" t="n">
+      <c r="C18" s="21" t="n">
         <f aca="false">$A18-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.02</v>
       </c>
-      <c r="D18" s="38" t="n">
+      <c r="D18" s="21" t="n">
         <f aca="false">$A18-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="E18" s="38" t="n">
+      <c r="E18" s="21" t="n">
         <f aca="false">$A18-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.14</v>
       </c>
-      <c r="F18" s="38" t="n">
+      <c r="F18" s="21" t="n">
         <f aca="false">$A18-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.2</v>
       </c>
-      <c r="G18" s="38" t="n">
+      <c r="G18" s="21" t="n">
         <f aca="false">$A18-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.35</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="38" t="n">
+      <c r="A19" s="21" t="n">
         <f aca="false">$A9</f>
         <v>0.2</v>
       </c>
-      <c r="B19" s="38" t="n">
+      <c r="B19" s="21" t="n">
         <f aca="false">$A19-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.14</v>
       </c>
-      <c r="C19" s="38" t="n">
+      <c r="C19" s="21" t="n">
         <f aca="false">$A19-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.08</v>
       </c>
-      <c r="D19" s="38" t="n">
+      <c r="D19" s="21" t="n">
         <f aca="false">$A19-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.02</v>
       </c>
-      <c r="E19" s="38" t="n">
+      <c r="E19" s="21" t="n">
         <f aca="false">$A19-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.04</v>
       </c>
-      <c r="F19" s="38" t="n">
+      <c r="F19" s="21" t="n">
         <f aca="false">$A19-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.1</v>
       </c>
-      <c r="G19" s="38" t="n">
+      <c r="G19" s="21" t="n">
         <f aca="false">$A19-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.25</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="38" t="n">
+      <c r="A20" s="21" t="n">
         <f aca="false">$A10</f>
         <v>0.3</v>
       </c>
-      <c r="B20" s="38" t="n">
+      <c r="B20" s="21" t="n">
         <f aca="false">$A20-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.24</v>
       </c>
-      <c r="C20" s="38" t="n">
+      <c r="C20" s="21" t="n">
         <f aca="false">$A20-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.18</v>
       </c>
-      <c r="D20" s="38" t="n">
+      <c r="D20" s="21" t="n">
         <f aca="false">$A20-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.12</v>
       </c>
-      <c r="E20" s="38" t="n">
+      <c r="E20" s="21" t="n">
         <f aca="false">$A20-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.06</v>
       </c>
-      <c r="F20" s="38" t="n">
+      <c r="F20" s="21" t="n">
         <f aca="false">$A20-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="G20" s="38" t="n">
+      <c r="G20" s="21" t="n">
         <f aca="false">$A20-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="38" t="n">
+      <c r="A21" s="21" t="n">
         <f aca="false">$A11</f>
         <v>0.5</v>
       </c>
-      <c r="B21" s="38" t="n">
+      <c r="B21" s="21" t="n">
         <f aca="false">$A21-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.44</v>
       </c>
-      <c r="C21" s="38" t="n">
+      <c r="C21" s="21" t="n">
         <f aca="false">$A21-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.38</v>
       </c>
-      <c r="D21" s="38" t="n">
+      <c r="D21" s="21" t="n">
         <f aca="false">$A21-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.32</v>
       </c>
-      <c r="E21" s="38" t="n">
+      <c r="E21" s="21" t="n">
         <f aca="false">$A21-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.26</v>
       </c>
-      <c r="F21" s="38" t="n">
+      <c r="F21" s="21" t="n">
         <f aca="false">$A21-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.2</v>
       </c>
-      <c r="G21" s="38" t="n">
+      <c r="G21" s="21" t="n">
         <f aca="false">$A21-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.05</v>
       </c>
@@ -3594,7 +3545,7 @@
       <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="40" t="n">
+      <c r="B5" s="29" t="n">
         <f aca="false">Supuestos!$B$17</f>
         <v>0.02</v>
       </c>
@@ -3609,7 +3560,7 @@
       <c r="A6" s="3" t="s">
         <v>125</v>
       </c>
-      <c r="B6" s="40" t="n">
+      <c r="B6" s="29" t="n">
         <f aca="false">Supuestos!$B$18</f>
         <v>0.1</v>
       </c>
@@ -3624,7 +3575,7 @@
       <c r="A7" s="3" t="s">
         <v>126</v>
       </c>
-      <c r="B7" s="40" t="n">
+      <c r="B7" s="29" t="n">
         <f aca="false">Supuestos!$B$15</f>
         <v>0.01</v>
       </c>
@@ -3639,7 +3590,7 @@
       <c r="A8" s="3" t="s">
         <v>127</v>
       </c>
-      <c r="B8" s="40" t="n">
+      <c r="B8" s="29" t="n">
         <f aca="false">Supuestos!$B$16</f>
         <v>0</v>
       </c>
@@ -3665,7 +3616,7 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="30" t="s">
         <v>129</v>
       </c>
       <c r="B10" s="3"/>
@@ -3690,15 +3641,15 @@
       <c r="A13" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B13" s="42" t="n">
+      <c r="B13" s="23" t="n">
         <f aca="false">1000*Supuestos!$B$8</f>
         <v>100</v>
       </c>
-      <c r="C13" s="42" t="n">
+      <c r="C13" s="23" t="n">
         <f aca="false">1000*Supuestos!$B$8</f>
         <v>100</v>
       </c>
-      <c r="D13" s="42" t="n">
+      <c r="D13" s="23" t="n">
         <f aca="false">1000*Supuestos!$B$8</f>
         <v>100</v>
       </c>
@@ -3707,15 +3658,15 @@
       <c r="A14" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B14" s="42" t="n">
+      <c r="B14" s="23" t="n">
         <f aca="false">1000*Supuestos!$B$40*B$5</f>
         <v>360</v>
       </c>
-      <c r="C14" s="42" t="n">
+      <c r="C14" s="23" t="n">
         <f aca="false">1000*Supuestos!$B$40*C$5</f>
         <v>45</v>
       </c>
-      <c r="D14" s="42" t="n">
+      <c r="D14" s="23" t="n">
         <f aca="false">1000*Supuestos!$B$40*D$5</f>
         <v>0</v>
       </c>
@@ -3724,15 +3675,15 @@
       <c r="A15" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="B15" s="42" t="n">
+      <c r="B15" s="23" t="n">
         <f aca="false">B13-B14</f>
         <v>-260</v>
       </c>
-      <c r="C15" s="42" t="n">
+      <c r="C15" s="23" t="n">
         <f aca="false">C13-C14</f>
         <v>55</v>
       </c>
-      <c r="D15" s="42" t="n">
+      <c r="D15" s="23" t="n">
         <f aca="false">D13-D14</f>
         <v>100</v>
       </c>
@@ -3741,15 +3692,15 @@
       <c r="A16" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B16" s="42" t="n">
+      <c r="B16" s="23" t="n">
         <f aca="false">MAX(0,B15)*B$6</f>
         <v>0</v>
       </c>
-      <c r="C16" s="42" t="n">
+      <c r="C16" s="23" t="n">
         <f aca="false">MAX(0,C15)*C$6</f>
         <v>11</v>
       </c>
-      <c r="D16" s="42" t="n">
+      <c r="D16" s="23" t="n">
         <f aca="false">MAX(0,D15)*D$6</f>
         <v>25</v>
       </c>
@@ -3758,15 +3709,15 @@
       <c r="A17" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="B17" s="42" t="n">
+      <c r="B17" s="23" t="n">
         <f aca="false">B$9</f>
         <v>0</v>
       </c>
-      <c r="C17" s="42" t="n">
+      <c r="C17" s="23" t="n">
         <f aca="false">C$9</f>
         <v>0</v>
       </c>
-      <c r="D17" s="42" t="n">
+      <c r="D17" s="23" t="n">
         <f aca="false">D$9</f>
         <v>0</v>
       </c>
@@ -3775,15 +3726,15 @@
       <c r="A18" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B18" s="36" t="n">
+      <c r="B18" s="24" t="n">
         <f aca="false">B15-B16-B17</f>
         <v>-260</v>
       </c>
-      <c r="C18" s="36" t="n">
+      <c r="C18" s="24" t="n">
         <f aca="false">C15-C16-C17</f>
         <v>44</v>
       </c>
-      <c r="D18" s="36" t="n">
+      <c r="D18" s="24" t="n">
         <f aca="false">D15-D16-D17</f>
         <v>75</v>
       </c>
@@ -3792,15 +3743,15 @@
       <c r="A19" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="B19" s="37" t="n">
+      <c r="B19" s="20" t="n">
         <f aca="false">B18/1000</f>
         <v>-0.26</v>
       </c>
-      <c r="C19" s="37" t="n">
+      <c r="C19" s="20" t="n">
         <f aca="false">C18/1000</f>
         <v>0.044</v>
       </c>
-      <c r="D19" s="37" t="n">
+      <c r="D19" s="20" t="n">
         <f aca="false">D18/1000</f>
         <v>0.075</v>
       </c>
@@ -3809,15 +3760,15 @@
       <c r="A20" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B20" s="36" t="n">
+      <c r="B20" s="24" t="n">
         <f aca="false">B14+B16+B17</f>
         <v>360</v>
       </c>
-      <c r="C20" s="36" t="n">
+      <c r="C20" s="24" t="n">
         <f aca="false">C14+C16+C17</f>
         <v>56</v>
       </c>
-      <c r="D20" s="36" t="n">
+      <c r="D20" s="24" t="n">
         <f aca="false">D14+D16+D17</f>
         <v>25</v>
       </c>
@@ -3826,15 +3777,15 @@
       <c r="A21" s="3" t="s">
         <v>139</v>
       </c>
-      <c r="B21" s="42" t="n">
+      <c r="B21" s="23" t="n">
         <f aca="false">Supuestos!$B$43</f>
         <v>16.2</v>
       </c>
-      <c r="C21" s="42" t="n">
+      <c r="C21" s="23" t="n">
         <f aca="false">Supuestos!$B$43</f>
         <v>16.2</v>
       </c>
-      <c r="D21" s="42" t="n">
+      <c r="D21" s="23" t="n">
         <f aca="false">Supuestos!$B$43</f>
         <v>16.2</v>
       </c>
@@ -3843,15 +3794,15 @@
       <c r="A22" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="B22" s="42" t="n">
+      <c r="B22" s="23" t="n">
         <f aca="false">B20-B21</f>
         <v>343.8</v>
       </c>
-      <c r="C22" s="42" t="n">
+      <c r="C22" s="23" t="n">
         <f aca="false">C20-C21</f>
         <v>39.8</v>
       </c>
-      <c r="D22" s="42" t="n">
+      <c r="D22" s="23" t="n">
         <f aca="false">D20-D21</f>
         <v>8.8</v>
       </c>
@@ -3860,15 +3811,15 @@
       <c r="A23" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="B23" s="38" t="n">
+      <c r="B23" s="21" t="n">
         <f aca="false">B14/1000</f>
         <v>0.36</v>
       </c>
-      <c r="C23" s="38" t="n">
+      <c r="C23" s="21" t="n">
         <f aca="false">C14/1000</f>
         <v>0.045</v>
       </c>
-      <c r="D23" s="38" t="n">
+      <c r="D23" s="21" t="n">
         <f aca="false">D14/1000</f>
         <v>0</v>
       </c>
@@ -3891,15 +3842,15 @@
       <c r="A26" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="B26" s="42" t="n">
+      <c r="B26" s="23" t="n">
         <f aca="false">1000*-0.1</f>
         <v>-100</v>
       </c>
-      <c r="C26" s="42" t="n">
+      <c r="C26" s="23" t="n">
         <f aca="false">1000*-0.1</f>
         <v>-100</v>
       </c>
-      <c r="D26" s="42" t="n">
+      <c r="D26" s="23" t="n">
         <f aca="false">1000*-0.1</f>
         <v>-100</v>
       </c>
@@ -3908,15 +3859,15 @@
       <c r="A27" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="B27" s="42" t="n">
+      <c r="B27" s="23" t="n">
         <f aca="false">1000*Supuestos!$B$40*B$5</f>
         <v>360</v>
       </c>
-      <c r="C27" s="42" t="n">
+      <c r="C27" s="23" t="n">
         <f aca="false">1000*Supuestos!$B$40*C$5</f>
         <v>45</v>
       </c>
-      <c r="D27" s="42" t="n">
+      <c r="D27" s="23" t="n">
         <f aca="false">1000*Supuestos!$B$40*D$5</f>
         <v>0</v>
       </c>
@@ -3925,15 +3876,15 @@
       <c r="A28" s="3" t="s">
         <v>136</v>
       </c>
-      <c r="B28" s="36" t="n">
+      <c r="B28" s="24" t="n">
         <f aca="false">B26-B27-B$9</f>
         <v>-460</v>
       </c>
-      <c r="C28" s="36" t="n">
+      <c r="C28" s="24" t="n">
         <f aca="false">C26-C27-C$9</f>
         <v>-145</v>
       </c>
-      <c r="D28" s="36" t="n">
+      <c r="D28" s="24" t="n">
         <f aca="false">D26-D27-D$9</f>
         <v>-100</v>
       </c>
@@ -3942,15 +3893,15 @@
       <c r="A29" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="B29" s="36" t="n">
+      <c r="B29" s="24" t="n">
         <f aca="false">B27+B$9</f>
         <v>360</v>
       </c>
-      <c r="C29" s="36" t="n">
+      <c r="C29" s="24" t="n">
         <f aca="false">C27+C$9</f>
         <v>45</v>
       </c>
-      <c r="D29" s="36" t="n">
+      <c r="D29" s="24" t="n">
         <f aca="false">D27+D$9</f>
         <v>0</v>
       </c>
@@ -3962,7 +3913,7 @@
       <c r="D30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="43" t="s">
+      <c r="A31" s="31" t="s">
         <v>143</v>
       </c>
       <c r="B31" s="3"/>
@@ -4027,27 +3978,27 @@
       <c r="A4" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="B4" s="44" t="n">
+      <c r="B4" s="32" t="n">
         <f aca="false">Escenarios!B4</f>
         <v>10</v>
       </c>
-      <c r="C4" s="44" t="n">
+      <c r="C4" s="32" t="n">
         <f aca="false">Escenarios!C4</f>
         <v>25</v>
       </c>
-      <c r="D4" s="44" t="n">
+      <c r="D4" s="32" t="n">
         <f aca="false">Escenarios!D4</f>
         <v>50</v>
       </c>
-      <c r="E4" s="44" t="n">
+      <c r="E4" s="32" t="n">
         <f aca="false">Escenarios!E4</f>
         <v>100</v>
       </c>
-      <c r="F4" s="44" t="n">
+      <c r="F4" s="32" t="n">
         <f aca="false">Escenarios!F4</f>
         <v>250</v>
       </c>
-      <c r="G4" s="44" t="n">
+      <c r="G4" s="32" t="n">
         <f aca="false">Escenarios!G4</f>
         <v>1000</v>
       </c>
@@ -4056,27 +4007,27 @@
       <c r="A5" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="B5" s="42" t="n">
+      <c r="B5" s="23" t="n">
         <f aca="false">B$4*Supuestos!$B$34</f>
         <v>10000</v>
       </c>
-      <c r="C5" s="42" t="n">
+      <c r="C5" s="23" t="n">
         <f aca="false">C$4*Supuestos!$B$34</f>
         <v>25000</v>
       </c>
-      <c r="D5" s="42" t="n">
+      <c r="D5" s="23" t="n">
         <f aca="false">D$4*Supuestos!$B$34</f>
         <v>50000</v>
       </c>
-      <c r="E5" s="42" t="n">
+      <c r="E5" s="23" t="n">
         <f aca="false">E$4*Supuestos!$B$34</f>
         <v>100000</v>
       </c>
-      <c r="F5" s="42" t="n">
+      <c r="F5" s="23" t="n">
         <f aca="false">F$4*Supuestos!$B$34</f>
         <v>250000</v>
       </c>
-      <c r="G5" s="42" t="n">
+      <c r="G5" s="23" t="n">
         <f aca="false">G$4*Supuestos!$B$34</f>
         <v>1000000</v>
       </c>
@@ -4085,27 +4036,27 @@
       <c r="A6" s="3" t="s">
         <v>97</v>
       </c>
-      <c r="B6" s="42" t="n">
+      <c r="B6" s="23" t="n">
         <f aca="false">B5*Supuestos!$B$35</f>
         <v>5000</v>
       </c>
-      <c r="C6" s="42" t="n">
+      <c r="C6" s="23" t="n">
         <f aca="false">C5*Supuestos!$B$35</f>
         <v>12500</v>
       </c>
-      <c r="D6" s="42" t="n">
+      <c r="D6" s="23" t="n">
         <f aca="false">D5*Supuestos!$B$35</f>
         <v>25000</v>
       </c>
-      <c r="E6" s="42" t="n">
+      <c r="E6" s="23" t="n">
         <f aca="false">E5*Supuestos!$B$35</f>
         <v>50000</v>
       </c>
-      <c r="F6" s="42" t="n">
+      <c r="F6" s="23" t="n">
         <f aca="false">F5*Supuestos!$B$35</f>
         <v>125000</v>
       </c>
-      <c r="G6" s="42" t="n">
+      <c r="G6" s="23" t="n">
         <f aca="false">G5*Supuestos!$B$35</f>
         <v>500000</v>
       </c>
@@ -4114,27 +4065,27 @@
       <c r="A7" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="B7" s="42" t="n">
+      <c r="B7" s="23" t="n">
         <f aca="false">B5-B6</f>
         <v>5000</v>
       </c>
-      <c r="C7" s="42" t="n">
+      <c r="C7" s="23" t="n">
         <f aca="false">C5-C6</f>
         <v>12500</v>
       </c>
-      <c r="D7" s="42" t="n">
+      <c r="D7" s="23" t="n">
         <f aca="false">D5-D6</f>
         <v>25000</v>
       </c>
-      <c r="E7" s="42" t="n">
+      <c r="E7" s="23" t="n">
         <f aca="false">E5-E6</f>
         <v>50000</v>
       </c>
-      <c r="F7" s="42" t="n">
+      <c r="F7" s="23" t="n">
         <f aca="false">F5-F6</f>
         <v>125000</v>
       </c>
-      <c r="G7" s="42" t="n">
+      <c r="G7" s="23" t="n">
         <f aca="false">G5-G6</f>
         <v>500000</v>
       </c>
@@ -4143,27 +4094,27 @@
       <c r="A8" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B8" s="42" t="n">
+      <c r="B8" s="23" t="n">
         <f aca="false">(B6*Alternativas!$C$7+B7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>450</v>
       </c>
-      <c r="C8" s="42" t="n">
+      <c r="C8" s="23" t="n">
         <f aca="false">(C6*Alternativas!$C$7+C7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>1125</v>
       </c>
-      <c r="D8" s="42" t="n">
+      <c r="D8" s="23" t="n">
         <f aca="false">(D6*Alternativas!$C$7+D7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>2250</v>
       </c>
-      <c r="E8" s="42" t="n">
+      <c r="E8" s="23" t="n">
         <f aca="false">(E6*Alternativas!$C$7+E7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>4500</v>
       </c>
-      <c r="F8" s="42" t="n">
+      <c r="F8" s="23" t="n">
         <f aca="false">(F6*Alternativas!$C$7+F7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>11250</v>
       </c>
-      <c r="G8" s="42" t="n">
+      <c r="G8" s="23" t="n">
         <f aca="false">(G6*Alternativas!$C$7+G7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>45000</v>
       </c>
@@ -4172,27 +4123,27 @@
       <c r="A9" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="B9" s="42" t="n">
+      <c r="B9" s="23" t="n">
         <f aca="false">B7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+B6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>82.5</v>
       </c>
-      <c r="C9" s="42" t="n">
+      <c r="C9" s="23" t="n">
         <f aca="false">C7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+C6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>206.25</v>
       </c>
-      <c r="D9" s="42" t="n">
+      <c r="D9" s="23" t="n">
         <f aca="false">D7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+D6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>412.5</v>
       </c>
-      <c r="E9" s="42" t="n">
+      <c r="E9" s="23" t="n">
         <f aca="false">E7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+E6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>825</v>
       </c>
-      <c r="F9" s="42" t="n">
+      <c r="F9" s="23" t="n">
         <f aca="false">F7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+F6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>2062.5</v>
       </c>
-      <c r="G9" s="42" t="n">
+      <c r="G9" s="23" t="n">
         <f aca="false">G7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+G6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>8250</v>
       </c>
@@ -4201,27 +4152,27 @@
       <c r="A10" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="B10" s="42" t="n">
+      <c r="B10" s="23" t="n">
         <f aca="false">B$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
-      <c r="C10" s="42" t="n">
+      <c r="C10" s="23" t="n">
         <f aca="false">C$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
-      <c r="D10" s="42" t="n">
+      <c r="D10" s="23" t="n">
         <f aca="false">D$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
-      <c r="E10" s="42" t="n">
+      <c r="E10" s="23" t="n">
         <f aca="false">E$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
-      <c r="F10" s="42" t="n">
+      <c r="F10" s="23" t="n">
         <f aca="false">F$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
-      <c r="G10" s="42" t="n">
+      <c r="G10" s="23" t="n">
         <f aca="false">G$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
@@ -4230,27 +4181,27 @@
       <c r="A11" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="B11" s="42" t="n">
+      <c r="B11" s="23" t="n">
         <f aca="false">SUM(B8:B10)</f>
         <v>532.5</v>
       </c>
-      <c r="C11" s="42" t="n">
+      <c r="C11" s="23" t="n">
         <f aca="false">SUM(C8:C10)</f>
         <v>1331.25</v>
       </c>
-      <c r="D11" s="42" t="n">
+      <c r="D11" s="23" t="n">
         <f aca="false">SUM(D8:D10)</f>
         <v>2662.5</v>
       </c>
-      <c r="E11" s="42" t="n">
+      <c r="E11" s="23" t="n">
         <f aca="false">SUM(E8:E10)</f>
         <v>5325</v>
       </c>
-      <c r="F11" s="42" t="n">
+      <c r="F11" s="23" t="n">
         <f aca="false">SUM(F8:F10)</f>
         <v>13312.5</v>
       </c>
-      <c r="G11" s="42" t="n">
+      <c r="G11" s="23" t="n">
         <f aca="false">SUM(G8:G10)</f>
         <v>53250</v>
       </c>
@@ -4259,27 +4210,27 @@
       <c r="A12" s="3" t="s">
         <v>88</v>
       </c>
-      <c r="B12" s="42" t="n">
+      <c r="B12" s="23" t="n">
         <f aca="false">Escenarios!B21</f>
         <v>471</v>
       </c>
-      <c r="C12" s="42" t="n">
+      <c r="C12" s="23" t="n">
         <f aca="false">Escenarios!C21</f>
         <v>714</v>
       </c>
-      <c r="D12" s="42" t="n">
+      <c r="D12" s="23" t="n">
         <f aca="false">Escenarios!D21</f>
         <v>1319</v>
       </c>
-      <c r="E12" s="42" t="n">
+      <c r="E12" s="23" t="n">
         <f aca="false">Escenarios!E21</f>
         <v>2129</v>
       </c>
-      <c r="F12" s="42" t="n">
+      <c r="F12" s="23" t="n">
         <f aca="false">Escenarios!F21</f>
         <v>4559</v>
       </c>
-      <c r="G12" s="42" t="n">
+      <c r="G12" s="23" t="n">
         <f aca="false">Escenarios!G21</f>
         <v>16709</v>
       </c>
@@ -4288,27 +4239,27 @@
       <c r="A13" s="3" t="s">
         <v>89</v>
       </c>
-      <c r="B13" s="36" t="n">
+      <c r="B13" s="24" t="n">
         <f aca="false">B11-B12</f>
         <v>61.5000000000001</v>
       </c>
-      <c r="C13" s="36" t="n">
+      <c r="C13" s="24" t="n">
         <f aca="false">C11-C12</f>
         <v>617.25</v>
       </c>
-      <c r="D13" s="36" t="n">
+      <c r="D13" s="24" t="n">
         <f aca="false">D11-D12</f>
         <v>1343.5</v>
       </c>
-      <c r="E13" s="36" t="n">
+      <c r="E13" s="24" t="n">
         <f aca="false">E11-E12</f>
         <v>3196</v>
       </c>
-      <c r="F13" s="36" t="n">
+      <c r="F13" s="24" t="n">
         <f aca="false">F11-F12</f>
         <v>8753.5</v>
       </c>
-      <c r="G13" s="36" t="n">
+      <c r="G13" s="24" t="n">
         <f aca="false">G11-G12</f>
         <v>36541</v>
       </c>
@@ -4317,27 +4268,27 @@
       <c r="A14" s="3" t="s">
         <v>113</v>
       </c>
-      <c r="B14" s="37" t="n">
+      <c r="B14" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
-      <c r="C14" s="37" t="n">
+      <c r="C14" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
-      <c r="D14" s="37" t="n">
+      <c r="D14" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
-      <c r="E14" s="37" t="n">
+      <c r="E14" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
-      <c r="F14" s="37" t="n">
+      <c r="F14" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
-      <c r="G14" s="37" t="n">
+      <c r="G14" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
@@ -4346,27 +4297,27 @@
       <c r="A15" s="3" t="s">
         <v>114</v>
       </c>
-      <c r="B15" s="37" t="n">
+      <c r="B15" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>
-      <c r="C15" s="37" t="n">
+      <c r="C15" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>
-      <c r="D15" s="37" t="n">
+      <c r="D15" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>
-      <c r="E15" s="37" t="n">
+      <c r="E15" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>
-      <c r="F15" s="37" t="n">
+      <c r="F15" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>
-      <c r="G15" s="37" t="n">
+      <c r="G15" s="20" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>

</xml_diff>

<commit_message>
modelo D final: 1% en tokens, 15% éxito externos, sin cuota, mínimo 300, billeteras separadas, costo on-chain optimizado; fijos compartidos fuera del incremental
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PW6Q8w1k9NaeArkk4QShv1
</commit_message>
<xml_diff>
--- a/docs/modelo_negocio_lloyd.xlsx
+++ b/docs/modelo_negocio_lloyd.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="149">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="174" uniqueCount="152">
   <si>
     <t xml:space="preserve">Lloyd's Tavern · supuestos del modelo</t>
   </si>
@@ -120,7 +120,7 @@
     <t xml:space="preserve">Servidores (Hetzner)</t>
   </si>
   <si>
-    <t xml:space="preserve">Estimado: el servidor del bot + el de la app. Ajustá con la factura real.</t>
+    <t xml:space="preserve">Incremental: el servidor del bot (CPX21). El de la app ya existía.</t>
   </si>
   <si>
     <t xml:space="preserve">Helius (RPC + webhooks)</t>
@@ -141,7 +141,7 @@
     <t xml:space="preserve">Claude (cerebro, sesiones de investigación, admin)</t>
   </si>
   <si>
-    <t xml:space="preserve">Hoy corre sobre la suscripción de Gastón. Poné acá la parte que le atribuís al bot.</t>
+    <t xml:space="preserve">Compartido: la suscripción de Claude y los servidores de Gastón existen con o sin el bot. Para saber si el bot se repaga, lo que cuenta es el costo incremental. Si querés cargárselo igual, poné acá el monto.</t>
   </si>
   <si>
     <t xml:space="preserve">X/Twitter API (cazador de tweets)</t>
@@ -207,7 +207,7 @@
     <t xml:space="preserve">Comisión de ejecución por operación con tokens (todos)</t>
   </si>
   <si>
-    <t xml:space="preserve">Gastón 29/10: el fee encubierto es fundamental; 5–10%/mes en memecoins no es grave. 1% solo sobre operaciones con tokens ≈ 9%/mes.</t>
+    <t xml:space="preserve">Gastón 29/10: el fee encubierto es fundamental; 5–10%/mes en memecoins no es grave. Embebida en el precio como 'fee included', como Jupiter y los bots de Telegram (0,5–1%).</t>
   </si>
   <si>
     <t xml:space="preserve">Parte del volumen que es operación con tokens (el resto es USDC/SOL)</t>
@@ -219,13 +219,13 @@
     <t xml:space="preserve">Externos · comisión de éxito sobre ganancia neta mensual (marca de agua)</t>
   </si>
   <si>
-    <t xml:space="preserve">Estándar de copy-trading y vaults: 15–25%.</t>
+    <t xml:space="preserve">Gastón 29/10: 15% y no más. Copy-trading y vaults cobran 15–25%.</t>
   </si>
   <si>
     <t xml:space="preserve">Externos · cuota de ingreso (US$), opcional</t>
   </si>
   <si>
-    <t xml:space="preserve">Gastón 29/10: sin cuota de ingreso; la gente no va a pagar para ver cómo funciona.</t>
+    <t xml:space="preserve">Gastón 29/10: sin cuota; la gente no va a pagar para ver cómo funciona. Queda en 0.</t>
   </si>
   <si>
     <t xml:space="preserve">Externos · meses que cubre la cuota de ingreso</t>
@@ -243,10 +243,16 @@
     <t xml:space="preserve">Gastón 29/10: mínimo de depósito US$300.</t>
   </si>
   <si>
+    <t xml:space="preserve">Costo on-chain + RPC por usuario por mes con el motor optimizado (US$)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hoy US$16 (180 operaciones × US$0,09). Si el motor no replica en las billeteras las operaciones de menos de US$20 y baja la prioridad fuera de momentos críticos, quedan ~60/mes ≈ US$6. Poné 16,2 para ver el caso sin optimizar.</t>
+  </si>
+  <si>
     <t xml:space="preserve">Billetera única (ómnibus) con libro interno: 1 = sí, 0 = una billetera por usuario</t>
   </si>
   <si>
-    <t xml:space="preserve">Gastón 29/10: billeteras separadas, cada uno ve su progreso.</t>
+    <t xml:space="preserve">Gastón 29/10: billeteras separadas, cada uno ve su progreso. Con ómnibus, Lloyd ejecuta UNA transacción por decisión para todos; el costo on-chain deja de crecer con los usuarios. Es lo que hace cualquier vault o bot de Telegram.</t>
   </si>
   <si>
     <t xml:space="preserve">Comisión de ejecución que paga cada cliente por mes (% de su capital)</t>
@@ -306,7 +312,10 @@
     <t xml:space="preserve">En un mes de −10%: lo que cobramos igual (ejecución + cuota)</t>
   </si>
   <si>
-    <t xml:space="preserve">Lectura: el negocio es un porcentaje del capital administrado, embebido en la ejecución. Los externos suman la comisión de éxito. La cuota de ingreso aporta poco: sirve como filtro, no como ingreso. Con billetera ómnibus, el costo on-chain es casi fijo y el margen crece con cada usuario.</t>
+    <t xml:space="preserve">Cada usuario se repaga: ingreso por usuario − costo on-chain por usuario</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lectura: cada usuario de US$300 deja ~US$27/mes de comisión de ejecución y cuesta ~US$6 de gas con el motor optimizado: se repaga solo. Los fijos propios del bot (servidor + Helius ≈ US$70) se cubren con 4 usuarios. La suscripción de Claude y los otros servidores existen con o sin el bot; si querés cargárselos, ponelos en Supuestos.</t>
   </si>
   <si>
     <t xml:space="preserve">Flujo mensual proyectado con el PRICING ACTUAL, por cantidad de usuarios</t>
@@ -478,7 +487,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="8">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.0%"/>
@@ -486,7 +495,8 @@
     <numFmt numFmtId="168" formatCode="\$#,##0.00;&quot;($&quot;#,##0.00\);\-"/>
     <numFmt numFmtId="169" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
     <numFmt numFmtId="170" formatCode="0.0\x"/>
-    <numFmt numFmtId="171" formatCode="#,##0"/>
+    <numFmt numFmtId="171" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
+    <numFmt numFmtId="172" formatCode="#,##0"/>
   </numFmts>
   <fonts count="13">
     <font>
@@ -629,7 +639,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="45">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -706,10 +716,78 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="166" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -718,7 +796,15 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -726,39 +812,11 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="169" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="171" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="172" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1249,7 +1307,7 @@
         <v>30</v>
       </c>
       <c r="B25" s="12" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="C25" s="7" t="s">
         <v>31</v>
@@ -1291,7 +1349,7 @@
         <v>37</v>
       </c>
       <c r="B29" s="12" t="n">
-        <v>200</v>
+        <v>0</v>
       </c>
       <c r="C29" s="7" t="s">
         <v>38</v>
@@ -1445,708 +1503,754 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:H34"/>
+  <dimension ref="A1:H36"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="52"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="1" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="60"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="52"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="60"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="19" t="s">
         <v>57</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
-      <c r="F1" s="3"/>
-      <c r="G1" s="3"/>
-      <c r="H1" s="3"/>
+      <c r="B1" s="20"/>
+      <c r="C1" s="20"/>
+      <c r="D1" s="20"/>
+      <c r="E1" s="20"/>
+      <c r="F1" s="20"/>
+      <c r="G1" s="20"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" customFormat="false" ht="43.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="19" t="s">
+      <c r="A2" s="21" t="s">
         <v>58</v>
       </c>
-      <c r="B2" s="19"/>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A3" s="3"/>
-      <c r="B3" s="3"/>
-      <c r="C3" s="3"/>
-      <c r="D3" s="3"/>
-      <c r="E3" s="3"/>
-      <c r="F3" s="3"/>
-      <c r="G3" s="3"/>
-      <c r="H3" s="3"/>
-    </row>
-    <row r="4" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
+      <c r="F2" s="21"/>
+      <c r="G2" s="21"/>
+      <c r="H2" s="21"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="20"/>
+      <c r="B3" s="20"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
+      <c r="E3" s="20"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
+      <c r="H3" s="20"/>
+    </row>
+    <row r="4" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="20" t="s">
         <v>59</v>
       </c>
-      <c r="B4" s="8" t="n">
+      <c r="B4" s="22" t="n">
         <v>0.01</v>
       </c>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
+      <c r="C4" s="20"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
       <c r="H4" s="7" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="3" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="20" t="s">
         <v>61</v>
       </c>
-      <c r="B5" s="8" t="n">
+      <c r="B5" s="22" t="n">
         <v>0.5</v>
       </c>
-      <c r="C5" s="3"/>
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-      <c r="G5" s="3"/>
+      <c r="C5" s="20"/>
+      <c r="D5" s="20"/>
+      <c r="E5" s="20"/>
+      <c r="F5" s="20"/>
+      <c r="G5" s="20"/>
       <c r="H5" s="7" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="20" t="s">
         <v>63</v>
       </c>
-      <c r="B6" s="8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="C6" s="3"/>
-      <c r="D6" s="3"/>
-      <c r="E6" s="3"/>
-      <c r="F6" s="3"/>
-      <c r="G6" s="3"/>
+      <c r="B6" s="22" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C6" s="20"/>
+      <c r="D6" s="20"/>
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="20"/>
       <c r="H6" s="7" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="3" t="s">
+    <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="20" t="s">
         <v>65</v>
       </c>
-      <c r="B7" s="12" t="n">
-        <v>0</v>
-      </c>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
+      <c r="B7" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="C7" s="20"/>
+      <c r="D7" s="20"/>
+      <c r="E7" s="20"/>
+      <c r="F7" s="20"/>
+      <c r="G7" s="20"/>
       <c r="H7" s="7" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="3" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="20" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="9" t="n">
+      <c r="B8" s="24" t="n">
         <v>6</v>
       </c>
-      <c r="C8" s="3"/>
-      <c r="D8" s="3"/>
-      <c r="E8" s="3"/>
-      <c r="F8" s="3"/>
-      <c r="G8" s="3"/>
+      <c r="C8" s="20"/>
+      <c r="D8" s="20"/>
+      <c r="E8" s="20"/>
+      <c r="F8" s="20"/>
+      <c r="G8" s="20"/>
       <c r="H8" s="7" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="3" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="20" t="s">
         <v>69</v>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="C9" s="3"/>
-      <c r="D9" s="3"/>
-      <c r="E9" s="3"/>
-      <c r="F9" s="3"/>
-      <c r="G9" s="3"/>
+      <c r="B9" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="C9" s="20"/>
+      <c r="D9" s="20"/>
+      <c r="E9" s="20"/>
+      <c r="F9" s="20"/>
+      <c r="G9" s="20"/>
       <c r="H9" s="7" t="s">
         <v>70</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="20" t="s">
         <v>43</v>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="23" t="n">
         <v>300</v>
       </c>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-      <c r="E10" s="3"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
       <c r="H10" s="7" t="s">
         <v>71</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="32.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A11" s="3" t="s">
+    <row r="11" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="B11" s="9" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
+      <c r="B11" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
       <c r="H11" s="7" t="s">
         <v>73</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="3" t="s">
+    <row r="12" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
         <v>74</v>
       </c>
-      <c r="B13" s="20" t="n">
+      <c r="B12" s="24" t="n">
+        <v>0</v>
+      </c>
+      <c r="C12" s="20"/>
+      <c r="D12" s="20"/>
+      <c r="E12" s="20"/>
+      <c r="F12" s="20"/>
+      <c r="G12" s="20"/>
+      <c r="H12" s="7" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B14" s="25" t="n">
         <f aca="false">Supuestos!$B$40*$B$5*$B$4</f>
         <v>0.09</v>
       </c>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A14" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="B14" s="20" t="n">
-        <f aca="false">Supuestos!$B$8-$B$13</f>
+      <c r="C14" s="20"/>
+      <c r="D14" s="20"/>
+      <c r="E14" s="20"/>
+      <c r="F14" s="20"/>
+      <c r="G14" s="20"/>
+      <c r="H14" s="20"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="B15" s="25" t="n">
+        <f aca="false">Supuestos!$B$8-$B$14</f>
         <v>0.01</v>
       </c>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="B15" s="20" t="n">
-        <f aca="false">Supuestos!$B$8-$B$13-MAX(0,Supuestos!$B$8-$B$13)*$B$6</f>
-        <v>0.00800000000000001</v>
-      </c>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-    </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="3" t="s">
-        <v>77</v>
-      </c>
-      <c r="B16" s="21" t="n">
-        <f aca="false">$B$13</f>
+      <c r="C15" s="20"/>
+      <c r="D15" s="20"/>
+      <c r="E15" s="20"/>
+      <c r="F15" s="20"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="20" t="s">
+        <v>78</v>
+      </c>
+      <c r="B16" s="25" t="n">
+        <f aca="false">Supuestos!$B$8-$B$14-MAX(0,Supuestos!$B$8-$B$14)*$B$6</f>
+        <v>0.00850000000000001</v>
+      </c>
+      <c r="C16" s="20"/>
+      <c r="D16" s="20"/>
+      <c r="E16" s="20"/>
+      <c r="F16" s="20"/>
+      <c r="G16" s="20"/>
+      <c r="H16" s="20"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="20" t="s">
+        <v>79</v>
+      </c>
+      <c r="B17" s="26" t="n">
+        <f aca="false">$B$14</f>
         <v>0.09</v>
       </c>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-    </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-    </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="B19" s="22" t="n">
+      <c r="C17" s="20"/>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="20"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="20"/>
+      <c r="B18" s="20"/>
+      <c r="C18" s="20"/>
+      <c r="D18" s="20"/>
+      <c r="E18" s="20"/>
+      <c r="F18" s="20"/>
+      <c r="G18" s="20"/>
+      <c r="H18" s="20"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="27" t="s">
+        <v>80</v>
+      </c>
+      <c r="B19" s="20"/>
+      <c r="C19" s="20"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="28" t="s">
+        <v>81</v>
+      </c>
+      <c r="B20" s="29" t="n">
         <v>10</v>
       </c>
-      <c r="C19" s="22" t="n">
+      <c r="C20" s="29" t="n">
         <v>25</v>
       </c>
-      <c r="D19" s="22" t="n">
+      <c r="D20" s="29" t="n">
         <v>50</v>
       </c>
-      <c r="E19" s="22" t="n">
+      <c r="E20" s="29" t="n">
         <v>100</v>
       </c>
-      <c r="F19" s="22" t="n">
+      <c r="F20" s="29" t="n">
         <v>250</v>
       </c>
-      <c r="G19" s="22" t="n">
+      <c r="G20" s="29" t="n">
         <v>1000</v>
       </c>
-      <c r="H19" s="3"/>
-    </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="3" t="s">
-        <v>80</v>
-      </c>
-      <c r="B20" s="23" t="n">
-        <f aca="false">B$19*$B$10</f>
+      <c r="H20" s="20"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="20" t="s">
+        <v>82</v>
+      </c>
+      <c r="B21" s="30" t="n">
+        <f aca="false">B$20*$B$10</f>
         <v>3000</v>
       </c>
-      <c r="C20" s="23" t="n">
-        <f aca="false">C$19*$B$10</f>
+      <c r="C21" s="30" t="n">
+        <f aca="false">C$20*$B$10</f>
         <v>7500</v>
       </c>
-      <c r="D20" s="23" t="n">
-        <f aca="false">D$19*$B$10</f>
+      <c r="D21" s="30" t="n">
+        <f aca="false">D$20*$B$10</f>
         <v>15000</v>
       </c>
-      <c r="E20" s="23" t="n">
-        <f aca="false">E$19*$B$10</f>
+      <c r="E21" s="30" t="n">
+        <f aca="false">E$20*$B$10</f>
         <v>30000</v>
       </c>
-      <c r="F20" s="23" t="n">
-        <f aca="false">F$19*$B$10</f>
+      <c r="F21" s="30" t="n">
+        <f aca="false">F$20*$B$10</f>
         <v>75000</v>
       </c>
-      <c r="G20" s="23" t="n">
-        <f aca="false">G$19*$B$10</f>
+      <c r="G21" s="30" t="n">
+        <f aca="false">G$20*$B$10</f>
         <v>300000</v>
       </c>
-      <c r="H20" s="3"/>
-    </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="3" t="s">
-        <v>81</v>
-      </c>
-      <c r="B21" s="23" t="n">
-        <f aca="false">B20*$B$13</f>
+      <c r="H21" s="20"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="20" t="s">
+        <v>83</v>
+      </c>
+      <c r="B22" s="30" t="n">
+        <f aca="false">B21*$B$14</f>
         <v>270</v>
       </c>
-      <c r="C21" s="23" t="n">
-        <f aca="false">C20*$B$13</f>
+      <c r="C22" s="30" t="n">
+        <f aca="false">C21*$B$14</f>
         <v>675</v>
       </c>
-      <c r="D21" s="23" t="n">
-        <f aca="false">D20*$B$13</f>
+      <c r="D22" s="30" t="n">
+        <f aca="false">D21*$B$14</f>
         <v>1350</v>
       </c>
-      <c r="E21" s="23" t="n">
-        <f aca="false">E20*$B$13</f>
+      <c r="E22" s="30" t="n">
+        <f aca="false">E21*$B$14</f>
         <v>2700</v>
       </c>
-      <c r="F21" s="23" t="n">
-        <f aca="false">F20*$B$13</f>
+      <c r="F22" s="30" t="n">
+        <f aca="false">F21*$B$14</f>
         <v>6750</v>
       </c>
-      <c r="G21" s="23" t="n">
-        <f aca="false">G20*$B$13</f>
+      <c r="G22" s="30" t="n">
+        <f aca="false">G21*$B$14</f>
         <v>27000</v>
       </c>
-      <c r="H21" s="3"/>
-    </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="B22" s="23" t="n">
-        <f aca="false">B20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+B20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>3</v>
-      </c>
-      <c r="C22" s="23" t="n">
-        <f aca="false">C20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+C20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>7.50000000000001</v>
-      </c>
-      <c r="D22" s="23" t="n">
-        <f aca="false">D20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+D20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>15</v>
-      </c>
-      <c r="E22" s="23" t="n">
-        <f aca="false">E20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+E20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>30</v>
-      </c>
-      <c r="F22" s="23" t="n">
-        <f aca="false">F20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+F20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
-        <v>75.0000000000001</v>
-      </c>
-      <c r="G22" s="23" t="n">
-        <f aca="false">G20*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$13)*$B$6+G20*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$13)*$B$9</f>
+      <c r="H22" s="20"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="20" t="s">
+        <v>84</v>
+      </c>
+      <c r="B23" s="30" t="n">
+        <f aca="false">B21*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$14)*$B$6+B21*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$14)*$B$9</f>
+        <v>2.25</v>
+      </c>
+      <c r="C23" s="30" t="n">
+        <f aca="false">C21*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$14)*$B$6+C21*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$14)*$B$9</f>
+        <v>5.62500000000001</v>
+      </c>
+      <c r="D23" s="30" t="n">
+        <f aca="false">D21*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$14)*$B$6+D21*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$14)*$B$9</f>
+        <v>11.25</v>
+      </c>
+      <c r="E23" s="30" t="n">
+        <f aca="false">E21*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$14)*$B$6+E21*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$14)*$B$9</f>
+        <v>22.5</v>
+      </c>
+      <c r="F23" s="30" t="n">
+        <f aca="false">F21*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$14)*$B$6+F21*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$14)*$B$9</f>
+        <v>56.2500000000001</v>
+      </c>
+      <c r="G23" s="30" t="n">
+        <f aca="false">G21*(1-Supuestos!$B$35)*MAX(0,Supuestos!$B$8-$B$14)*$B$6+G21*Supuestos!$B$35*MAX(0,Supuestos!$B$8-$B$14)*$B$9</f>
+        <v>225</v>
+      </c>
+      <c r="H23" s="20"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="20" t="s">
+        <v>85</v>
+      </c>
+      <c r="B24" s="30" t="n">
+        <f aca="false">B$20*(1-Supuestos!$B$35)*$B$7/$B$8</f>
+        <v>0</v>
+      </c>
+      <c r="C24" s="30" t="n">
+        <f aca="false">C$20*(1-Supuestos!$B$35)*$B$7/$B$8</f>
+        <v>0</v>
+      </c>
+      <c r="D24" s="30" t="n">
+        <f aca="false">D$20*(1-Supuestos!$B$35)*$B$7/$B$8</f>
+        <v>0</v>
+      </c>
+      <c r="E24" s="30" t="n">
+        <f aca="false">E$20*(1-Supuestos!$B$35)*$B$7/$B$8</f>
+        <v>0</v>
+      </c>
+      <c r="F24" s="30" t="n">
+        <f aca="false">F$20*(1-Supuestos!$B$35)*$B$7/$B$8</f>
+        <v>0</v>
+      </c>
+      <c r="G24" s="30" t="n">
+        <f aca="false">G$20*(1-Supuestos!$B$35)*$B$7/$B$8</f>
+        <v>0</v>
+      </c>
+      <c r="H24" s="20"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="20" t="s">
+        <v>86</v>
+      </c>
+      <c r="B25" s="31" t="n">
+        <f aca="false">SUM(B22:B24)</f>
+        <v>272.25</v>
+      </c>
+      <c r="C25" s="31" t="n">
+        <f aca="false">SUM(C22:C24)</f>
+        <v>680.625</v>
+      </c>
+      <c r="D25" s="31" t="n">
+        <f aca="false">SUM(D22:D24)</f>
+        <v>1361.25</v>
+      </c>
+      <c r="E25" s="31" t="n">
+        <f aca="false">SUM(E22:E24)</f>
+        <v>2722.5</v>
+      </c>
+      <c r="F25" s="31" t="n">
+        <f aca="false">SUM(F22:F24)</f>
+        <v>6806.25</v>
+      </c>
+      <c r="G25" s="31" t="n">
+        <f aca="false">SUM(G22:G24)</f>
+        <v>27225</v>
+      </c>
+      <c r="H25" s="20"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="20" t="s">
+        <v>87</v>
+      </c>
+      <c r="B26" s="30" t="n">
+        <f aca="false">IF($B$12=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),B$20*$B$11)</f>
+        <v>60</v>
+      </c>
+      <c r="C26" s="30" t="n">
+        <f aca="false">IF($B$12=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),C$20*$B$11)</f>
+        <v>150</v>
+      </c>
+      <c r="D26" s="30" t="n">
+        <f aca="false">IF($B$12=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),D$20*$B$11)</f>
         <v>300</v>
       </c>
-      <c r="H22" s="3"/>
-    </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A23" s="3" t="s">
-        <v>83</v>
-      </c>
-      <c r="B23" s="23" t="n">
-        <f aca="false">B$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>0</v>
-      </c>
-      <c r="C23" s="23" t="n">
-        <f aca="false">C$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>0</v>
-      </c>
-      <c r="D23" s="23" t="n">
-        <f aca="false">D$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>0</v>
-      </c>
-      <c r="E23" s="23" t="n">
-        <f aca="false">E$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>0</v>
-      </c>
-      <c r="F23" s="23" t="n">
-        <f aca="false">F$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>0</v>
-      </c>
-      <c r="G23" s="23" t="n">
-        <f aca="false">G$19*(1-Supuestos!$B$35)*$B$7/$B$8</f>
-        <v>0</v>
-      </c>
-      <c r="H23" s="3"/>
-    </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A24" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B24" s="24" t="n">
-        <f aca="false">SUM(B21:B23)</f>
-        <v>273</v>
-      </c>
-      <c r="C24" s="24" t="n">
-        <f aca="false">SUM(C21:C23)</f>
-        <v>682.5</v>
-      </c>
-      <c r="D24" s="24" t="n">
-        <f aca="false">SUM(D21:D23)</f>
-        <v>1365</v>
-      </c>
-      <c r="E24" s="24" t="n">
-        <f aca="false">SUM(E21:E23)</f>
-        <v>2730</v>
-      </c>
-      <c r="F24" s="24" t="n">
-        <f aca="false">SUM(F21:F23)</f>
-        <v>6825</v>
-      </c>
-      <c r="G24" s="24" t="n">
-        <f aca="false">SUM(G21:G23)</f>
-        <v>27300</v>
-      </c>
-      <c r="H24" s="3"/>
-    </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A25" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="B25" s="23" t="n">
-        <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),B$19*Supuestos!$B$43)</f>
-        <v>162</v>
-      </c>
-      <c r="C25" s="23" t="n">
-        <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),C$19*Supuestos!$B$43)</f>
-        <v>405</v>
-      </c>
-      <c r="D25" s="23" t="n">
-        <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),D$19*Supuestos!$B$43)</f>
-        <v>810</v>
-      </c>
-      <c r="E25" s="23" t="n">
-        <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),E$19*Supuestos!$B$43)</f>
-        <v>1620</v>
-      </c>
-      <c r="F25" s="23" t="n">
-        <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),F$19*Supuestos!$B$43)</f>
-        <v>4050</v>
-      </c>
-      <c r="G25" s="23" t="n">
-        <f aca="false">IF($B$11=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),G$19*Supuestos!$B$43)</f>
-        <v>16200</v>
-      </c>
-      <c r="H25" s="3"/>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A26" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B26" s="23" t="n">
-        <f aca="false">IF(B$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
+      <c r="E26" s="30" t="n">
+        <f aca="false">IF($B$12=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),E$20*$B$11)</f>
+        <v>600</v>
+      </c>
+      <c r="F26" s="30" t="n">
+        <f aca="false">IF($B$12=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),F$20*$B$11)</f>
+        <v>1500</v>
+      </c>
+      <c r="G26" s="30" t="n">
+        <f aca="false">IF($B$12=1,Supuestos!$B$39*(Supuestos!$B$21+Supuestos!$B$22),G$20*$B$11)</f>
+        <v>6000</v>
+      </c>
+      <c r="H26" s="20"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="B27" s="30" t="n">
+        <f aca="false">IF(B$20&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>49</v>
       </c>
-      <c r="C26" s="23" t="n">
-        <f aca="false">IF(C$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
+      <c r="C27" s="30" t="n">
+        <f aca="false">IF(C$20&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>49</v>
       </c>
-      <c r="D26" s="23" t="n">
-        <f aca="false">IF(D$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
+      <c r="D27" s="30" t="n">
+        <f aca="false">IF(D$20&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="E26" s="23" t="n">
-        <f aca="false">IF(E$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
+      <c r="E27" s="30" t="n">
+        <f aca="false">IF(E$20&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="F26" s="23" t="n">
-        <f aca="false">IF(F$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
+      <c r="F27" s="30" t="n">
+        <f aca="false">IF(F$20&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="G26" s="23" t="n">
-        <f aca="false">IF(G$19&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
+      <c r="G27" s="30" t="n">
+        <f aca="false">IF(G$20&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="H26" s="3"/>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A27" s="3" t="s">
-        <v>87</v>
-      </c>
-      <c r="B27" s="23" t="n">
+      <c r="H27" s="20"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="20" t="s">
+        <v>89</v>
+      </c>
+      <c r="B28" s="30" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="C27" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="C28" s="30" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="D27" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="D28" s="30" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="E27" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="E28" s="30" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="F27" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="F28" s="30" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="G27" s="23" t="n">
+        <v>35</v>
+      </c>
+      <c r="G28" s="30" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="H27" s="3"/>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A28" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B28" s="24" t="n">
-        <f aca="false">SUM(B25:B27)</f>
-        <v>471</v>
-      </c>
-      <c r="C28" s="24" t="n">
-        <f aca="false">SUM(C25:C27)</f>
-        <v>714</v>
-      </c>
-      <c r="D28" s="24" t="n">
-        <f aca="false">SUM(D25:D27)</f>
-        <v>1319</v>
-      </c>
-      <c r="E28" s="24" t="n">
-        <f aca="false">SUM(E25:E27)</f>
-        <v>2129</v>
-      </c>
-      <c r="F28" s="24" t="n">
-        <f aca="false">SUM(F25:F27)</f>
-        <v>4559</v>
-      </c>
-      <c r="G28" s="24" t="n">
-        <f aca="false">SUM(G25:G27)</f>
-        <v>16709</v>
-      </c>
-      <c r="H28" s="3"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A29" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="B29" s="24" t="n">
-        <f aca="false">B24-B28</f>
-        <v>-198</v>
-      </c>
-      <c r="C29" s="24" t="n">
-        <f aca="false">C24-C28</f>
-        <v>-31.4999999999999</v>
-      </c>
-      <c r="D29" s="24" t="n">
-        <f aca="false">D24-D28</f>
-        <v>46.0000000000002</v>
-      </c>
-      <c r="E29" s="24" t="n">
-        <f aca="false">E24-E28</f>
-        <v>601.000000000001</v>
-      </c>
-      <c r="F29" s="24" t="n">
-        <f aca="false">F24-F28</f>
-        <v>2266</v>
-      </c>
-      <c r="G29" s="24" t="n">
-        <f aca="false">G24-G28</f>
-        <v>10591</v>
-      </c>
-      <c r="H29" s="3"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A30" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H28" s="20"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="20" t="s">
         <v>90</v>
       </c>
-      <c r="B30" s="23" t="n">
-        <f aca="false">B29*12</f>
-        <v>-2376</v>
-      </c>
-      <c r="C30" s="23" t="n">
-        <f aca="false">C29*12</f>
-        <v>-377.999999999999</v>
-      </c>
-      <c r="D30" s="23" t="n">
-        <f aca="false">D29*12</f>
-        <v>552.000000000003</v>
-      </c>
-      <c r="E30" s="23" t="n">
-        <f aca="false">E29*12</f>
-        <v>7212.00000000001</v>
-      </c>
-      <c r="F30" s="23" t="n">
-        <f aca="false">F29*12</f>
-        <v>27192</v>
-      </c>
-      <c r="G30" s="23" t="n">
-        <f aca="false">G29*12</f>
-        <v>127092</v>
-      </c>
-      <c r="H30" s="3"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="3" t="s">
+      <c r="B29" s="31" t="n">
+        <f aca="false">SUM(B26:B28)</f>
+        <v>144</v>
+      </c>
+      <c r="C29" s="31" t="n">
+        <f aca="false">SUM(C26:C28)</f>
+        <v>234</v>
+      </c>
+      <c r="D29" s="31" t="n">
+        <f aca="false">SUM(D26:D28)</f>
+        <v>584</v>
+      </c>
+      <c r="E29" s="31" t="n">
+        <f aca="false">SUM(E26:E28)</f>
+        <v>884</v>
+      </c>
+      <c r="F29" s="31" t="n">
+        <f aca="false">SUM(F26:F28)</f>
+        <v>1784</v>
+      </c>
+      <c r="G29" s="31" t="n">
+        <f aca="false">SUM(G26:G28)</f>
+        <v>6284</v>
+      </c>
+      <c r="H29" s="20"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="20" t="s">
         <v>91</v>
       </c>
-      <c r="B31" s="23" t="n">
-        <f aca="false">IF(B$19=0,0,B24/B$19)</f>
-        <v>27.3</v>
-      </c>
-      <c r="C31" s="23" t="n">
-        <f aca="false">IF(C$19=0,0,C24/C$19)</f>
-        <v>27.3</v>
-      </c>
-      <c r="D31" s="23" t="n">
-        <f aca="false">IF(D$19=0,0,D24/D$19)</f>
-        <v>27.3</v>
-      </c>
-      <c r="E31" s="23" t="n">
-        <f aca="false">IF(E$19=0,0,E24/E$19)</f>
-        <v>27.3</v>
-      </c>
-      <c r="F31" s="23" t="n">
-        <f aca="false">IF(F$19=0,0,F24/F$19)</f>
-        <v>27.3</v>
-      </c>
-      <c r="G31" s="23" t="n">
-        <f aca="false">IF(G$19=0,0,G24/G$19)</f>
-        <v>27.3</v>
-      </c>
-      <c r="H31" s="3"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A32" s="3" t="s">
+      <c r="B30" s="31" t="n">
+        <f aca="false">B25-B29</f>
+        <v>128.25</v>
+      </c>
+      <c r="C30" s="31" t="n">
+        <f aca="false">C25-C29</f>
+        <v>446.625</v>
+      </c>
+      <c r="D30" s="31" t="n">
+        <f aca="false">D25-D29</f>
+        <v>777.25</v>
+      </c>
+      <c r="E30" s="31" t="n">
+        <f aca="false">E25-E29</f>
+        <v>1838.5</v>
+      </c>
+      <c r="F30" s="31" t="n">
+        <f aca="false">F25-F29</f>
+        <v>5022.25</v>
+      </c>
+      <c r="G30" s="31" t="n">
+        <f aca="false">G25-G29</f>
+        <v>20941</v>
+      </c>
+      <c r="H30" s="20"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="20" t="s">
         <v>92</v>
       </c>
-      <c r="B32" s="23" t="n">
-        <f aca="false">B21+B23</f>
+      <c r="B31" s="30" t="n">
+        <f aca="false">B30*12</f>
+        <v>1539</v>
+      </c>
+      <c r="C31" s="30" t="n">
+        <f aca="false">C30*12</f>
+        <v>5359.5</v>
+      </c>
+      <c r="D31" s="30" t="n">
+        <f aca="false">D30*12</f>
+        <v>9327</v>
+      </c>
+      <c r="E31" s="30" t="n">
+        <f aca="false">E30*12</f>
+        <v>22062</v>
+      </c>
+      <c r="F31" s="30" t="n">
+        <f aca="false">F30*12</f>
+        <v>60267</v>
+      </c>
+      <c r="G31" s="30" t="n">
+        <f aca="false">G30*12</f>
+        <v>251292</v>
+      </c>
+      <c r="H31" s="20"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="B32" s="30" t="n">
+        <f aca="false">IF(B$20=0,0,B25/B$20)</f>
+        <v>27.225</v>
+      </c>
+      <c r="C32" s="30" t="n">
+        <f aca="false">IF(C$20=0,0,C25/C$20)</f>
+        <v>27.225</v>
+      </c>
+      <c r="D32" s="30" t="n">
+        <f aca="false">IF(D$20=0,0,D25/D$20)</f>
+        <v>27.225</v>
+      </c>
+      <c r="E32" s="30" t="n">
+        <f aca="false">IF(E$20=0,0,E25/E$20)</f>
+        <v>27.225</v>
+      </c>
+      <c r="F32" s="30" t="n">
+        <f aca="false">IF(F$20=0,0,F25/F$20)</f>
+        <v>27.225</v>
+      </c>
+      <c r="G32" s="30" t="n">
+        <f aca="false">IF(G$20=0,0,G25/G$20)</f>
+        <v>27.225</v>
+      </c>
+      <c r="H32" s="20"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="B33" s="30" t="n">
+        <f aca="false">B22+B24</f>
         <v>270</v>
       </c>
-      <c r="C32" s="23" t="n">
-        <f aca="false">C21+C23</f>
+      <c r="C33" s="30" t="n">
+        <f aca="false">C22+C24</f>
         <v>675</v>
       </c>
-      <c r="D32" s="23" t="n">
-        <f aca="false">D21+D23</f>
+      <c r="D33" s="30" t="n">
+        <f aca="false">D22+D24</f>
         <v>1350</v>
       </c>
-      <c r="E32" s="23" t="n">
-        <f aca="false">E21+E23</f>
+      <c r="E33" s="30" t="n">
+        <f aca="false">E22+E24</f>
         <v>2700</v>
       </c>
-      <c r="F32" s="23" t="n">
-        <f aca="false">F21+F23</f>
+      <c r="F33" s="30" t="n">
+        <f aca="false">F22+F24</f>
         <v>6750</v>
       </c>
-      <c r="G32" s="23" t="n">
-        <f aca="false">G21+G23</f>
+      <c r="G33" s="30" t="n">
+        <f aca="false">G22+G24</f>
         <v>27000</v>
       </c>
-      <c r="H32" s="3"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-    </row>
-    <row r="34" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A34" s="25" t="s">
-        <v>93</v>
-      </c>
-      <c r="B34" s="25"/>
-      <c r="C34" s="25"/>
-      <c r="D34" s="25"/>
-      <c r="E34" s="25"/>
-      <c r="F34" s="25"/>
-      <c r="G34" s="25"/>
-      <c r="H34" s="25"/>
+      <c r="H33" s="20"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="B34" s="30" t="n">
+        <f aca="false">B32-$B$11</f>
+        <v>21.225</v>
+      </c>
+      <c r="C34" s="30" t="n">
+        <f aca="false">C32-$B$11</f>
+        <v>21.225</v>
+      </c>
+      <c r="D34" s="30" t="n">
+        <f aca="false">D32-$B$11</f>
+        <v>21.225</v>
+      </c>
+      <c r="E34" s="30" t="n">
+        <f aca="false">E32-$B$11</f>
+        <v>21.225</v>
+      </c>
+      <c r="F34" s="30" t="n">
+        <f aca="false">F32-$B$11</f>
+        <v>21.225</v>
+      </c>
+      <c r="G34" s="30" t="n">
+        <f aca="false">G32-$B$11</f>
+        <v>21.225</v>
+      </c>
+      <c r="H34" s="20"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="20"/>
+      <c r="B35" s="20"/>
+      <c r="C35" s="20"/>
+      <c r="D35" s="20"/>
+      <c r="E35" s="20"/>
+      <c r="F35" s="20"/>
+      <c r="G35" s="20"/>
+      <c r="H35" s="20"/>
+    </row>
+    <row r="36" customFormat="false" ht="39.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="32" t="s">
+        <v>96</v>
+      </c>
+      <c r="B36" s="32"/>
+      <c r="C36" s="32"/>
+      <c r="D36" s="32"/>
+      <c r="E36" s="32"/>
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32"/>
     </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A2:H2"/>
-    <mergeCell ref="A34:H34"/>
+    <mergeCell ref="A36:H36"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2172,7 +2276,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2183,7 +2287,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2203,139 +2307,139 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="22" t="n">
+        <v>81</v>
+      </c>
+      <c r="B4" s="33" t="n">
         <v>10</v>
       </c>
-      <c r="C4" s="22" t="n">
+      <c r="C4" s="33" t="n">
         <v>25</v>
       </c>
-      <c r="D4" s="22" t="n">
+      <c r="D4" s="33" t="n">
         <v>50</v>
       </c>
-      <c r="E4" s="22" t="n">
+      <c r="E4" s="33" t="n">
         <v>100</v>
       </c>
-      <c r="F4" s="22" t="n">
+      <c r="F4" s="33" t="n">
         <v>250</v>
       </c>
-      <c r="G4" s="22" t="n">
+      <c r="G4" s="33" t="n">
         <v>1000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" s="26" t="n">
+        <v>99</v>
+      </c>
+      <c r="B5" s="34" t="n">
         <f aca="false">B$4*Supuestos!$B$34</f>
         <v>10000</v>
       </c>
-      <c r="C5" s="26" t="n">
+      <c r="C5" s="34" t="n">
         <f aca="false">C$4*Supuestos!$B$34</f>
         <v>25000</v>
       </c>
-      <c r="D5" s="26" t="n">
+      <c r="D5" s="34" t="n">
         <f aca="false">D$4*Supuestos!$B$34</f>
         <v>50000</v>
       </c>
-      <c r="E5" s="26" t="n">
+      <c r="E5" s="34" t="n">
         <f aca="false">E$4*Supuestos!$B$34</f>
         <v>100000</v>
       </c>
-      <c r="F5" s="26" t="n">
+      <c r="F5" s="34" t="n">
         <f aca="false">F$4*Supuestos!$B$34</f>
         <v>250000</v>
       </c>
-      <c r="G5" s="26" t="n">
+      <c r="G5" s="34" t="n">
         <f aca="false">G$4*Supuestos!$B$34</f>
         <v>1000000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B6" s="26" t="n">
+        <v>100</v>
+      </c>
+      <c r="B6" s="34" t="n">
         <f aca="false">B5*Supuestos!$B$35</f>
         <v>5000</v>
       </c>
-      <c r="C6" s="26" t="n">
+      <c r="C6" s="34" t="n">
         <f aca="false">C5*Supuestos!$B$35</f>
         <v>12500</v>
       </c>
-      <c r="D6" s="26" t="n">
+      <c r="D6" s="34" t="n">
         <f aca="false">D5*Supuestos!$B$35</f>
         <v>25000</v>
       </c>
-      <c r="E6" s="26" t="n">
+      <c r="E6" s="34" t="n">
         <f aca="false">E5*Supuestos!$B$35</f>
         <v>50000</v>
       </c>
-      <c r="F6" s="26" t="n">
+      <c r="F6" s="34" t="n">
         <f aca="false">F5*Supuestos!$B$35</f>
         <v>125000</v>
       </c>
-      <c r="G6" s="26" t="n">
+      <c r="G6" s="34" t="n">
         <f aca="false">G5*Supuestos!$B$35</f>
         <v>500000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B7" s="26" t="n">
+        <v>101</v>
+      </c>
+      <c r="B7" s="34" t="n">
         <f aca="false">B5-B6</f>
         <v>5000</v>
       </c>
-      <c r="C7" s="26" t="n">
+      <c r="C7" s="34" t="n">
         <f aca="false">C5-C6</f>
         <v>12500</v>
       </c>
-      <c r="D7" s="26" t="n">
+      <c r="D7" s="34" t="n">
         <f aca="false">D5-D6</f>
         <v>25000</v>
       </c>
-      <c r="E7" s="26" t="n">
+      <c r="E7" s="34" t="n">
         <f aca="false">E5-E6</f>
         <v>50000</v>
       </c>
-      <c r="F7" s="26" t="n">
+      <c r="F7" s="34" t="n">
         <f aca="false">F5-F6</f>
         <v>125000</v>
       </c>
-      <c r="G7" s="26" t="n">
+      <c r="G7" s="34" t="n">
         <f aca="false">G5-G6</f>
         <v>500000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>99</v>
-      </c>
-      <c r="B8" s="27" t="n">
+        <v>102</v>
+      </c>
+      <c r="B8" s="35" t="n">
         <f aca="false">B$4*Supuestos!$B$39</f>
         <v>1800</v>
       </c>
-      <c r="C8" s="27" t="n">
+      <c r="C8" s="35" t="n">
         <f aca="false">C$4*Supuestos!$B$39</f>
         <v>4500</v>
       </c>
-      <c r="D8" s="27" t="n">
+      <c r="D8" s="35" t="n">
         <f aca="false">D$4*Supuestos!$B$39</f>
         <v>9000</v>
       </c>
-      <c r="E8" s="27" t="n">
+      <c r="E8" s="35" t="n">
         <f aca="false">E$4*Supuestos!$B$39</f>
         <v>18000</v>
       </c>
-      <c r="F8" s="27" t="n">
+      <c r="F8" s="35" t="n">
         <f aca="false">F$4*Supuestos!$B$39</f>
         <v>45000</v>
       </c>
-      <c r="G8" s="27" t="n">
+      <c r="G8" s="35" t="n">
         <f aca="false">G$4*Supuestos!$B$39</f>
         <v>180000</v>
       </c>
@@ -2351,7 +2455,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -2362,145 +2466,145 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>101</v>
-      </c>
-      <c r="B11" s="26" t="n">
+        <v>104</v>
+      </c>
+      <c r="B11" s="34" t="n">
         <f aca="false">B6*Supuestos!$B$41</f>
         <v>900</v>
       </c>
-      <c r="C11" s="26" t="n">
+      <c r="C11" s="34" t="n">
         <f aca="false">C6*Supuestos!$B$41</f>
         <v>2250</v>
       </c>
-      <c r="D11" s="26" t="n">
+      <c r="D11" s="34" t="n">
         <f aca="false">D6*Supuestos!$B$41</f>
         <v>4500</v>
       </c>
-      <c r="E11" s="26" t="n">
+      <c r="E11" s="34" t="n">
         <f aca="false">E6*Supuestos!$B$41</f>
         <v>9000</v>
       </c>
-      <c r="F11" s="26" t="n">
+      <c r="F11" s="34" t="n">
         <f aca="false">F6*Supuestos!$B$41</f>
         <v>22500</v>
       </c>
-      <c r="G11" s="26" t="n">
+      <c r="G11" s="34" t="n">
         <f aca="false">G6*Supuestos!$B$41</f>
         <v>90000</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>102</v>
-      </c>
-      <c r="B12" s="26" t="n">
+        <v>105</v>
+      </c>
+      <c r="B12" s="34" t="n">
         <f aca="false">B7*Supuestos!$B$42</f>
         <v>1800</v>
       </c>
-      <c r="C12" s="26" t="n">
+      <c r="C12" s="34" t="n">
         <f aca="false">C7*Supuestos!$B$42</f>
         <v>4500</v>
       </c>
-      <c r="D12" s="26" t="n">
+      <c r="D12" s="34" t="n">
         <f aca="false">D7*Supuestos!$B$42</f>
         <v>9000</v>
       </c>
-      <c r="E12" s="26" t="n">
+      <c r="E12" s="34" t="n">
         <f aca="false">E7*Supuestos!$B$42</f>
         <v>18000</v>
       </c>
-      <c r="F12" s="26" t="n">
+      <c r="F12" s="34" t="n">
         <f aca="false">F7*Supuestos!$B$42</f>
         <v>45000</v>
       </c>
-      <c r="G12" s="26" t="n">
+      <c r="G12" s="34" t="n">
         <f aca="false">G7*Supuestos!$B$42</f>
         <v>180000</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>103</v>
-      </c>
-      <c r="B13" s="26" t="n">
+        <v>106</v>
+      </c>
+      <c r="B13" s="34" t="n">
         <f aca="false">B7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
-      <c r="C13" s="26" t="n">
+      <c r="C13" s="34" t="n">
         <f aca="false">C7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
-      <c r="D13" s="26" t="n">
+      <c r="D13" s="34" t="n">
         <f aca="false">D7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
-      <c r="E13" s="26" t="n">
+      <c r="E13" s="34" t="n">
         <f aca="false">E7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
-      <c r="F13" s="26" t="n">
+      <c r="F13" s="34" t="n">
         <f aca="false">F7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
-      <c r="G13" s="26" t="n">
+      <c r="G13" s="34" t="n">
         <f aca="false">G7*MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
         <v>0</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>104</v>
-      </c>
-      <c r="B14" s="26" t="n">
+        <v>107</v>
+      </c>
+      <c r="B14" s="34" t="n">
         <f aca="false">B6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="C14" s="26" t="n">
+      <c r="C14" s="34" t="n">
         <f aca="false">C6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="D14" s="26" t="n">
+      <c r="D14" s="34" t="n">
         <f aca="false">D6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="E14" s="26" t="n">
+      <c r="E14" s="34" t="n">
         <f aca="false">E6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="F14" s="26" t="n">
+      <c r="F14" s="34" t="n">
         <f aca="false">F6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="G14" s="26" t="n">
+      <c r="G14" s="34" t="n">
         <f aca="false">G6*MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B15" s="26" t="n">
+        <v>86</v>
+      </c>
+      <c r="B15" s="34" t="n">
         <f aca="false">SUM(B11:B14)</f>
         <v>2700</v>
       </c>
-      <c r="C15" s="26" t="n">
+      <c r="C15" s="34" t="n">
         <f aca="false">SUM(C11:C14)</f>
         <v>6750</v>
       </c>
-      <c r="D15" s="26" t="n">
+      <c r="D15" s="34" t="n">
         <f aca="false">SUM(D11:D14)</f>
         <v>13500</v>
       </c>
-      <c r="E15" s="26" t="n">
+      <c r="E15" s="34" t="n">
         <f aca="false">SUM(E11:E14)</f>
         <v>27000</v>
       </c>
-      <c r="F15" s="26" t="n">
+      <c r="F15" s="34" t="n">
         <f aca="false">SUM(F11:F14)</f>
         <v>67500</v>
       </c>
-      <c r="G15" s="26" t="n">
+      <c r="G15" s="34" t="n">
         <f aca="false">SUM(G11:G14)</f>
         <v>270000</v>
       </c>
@@ -2516,7 +2620,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="B17" s="3"/>
       <c r="C17" s="3"/>
@@ -2527,118 +2631,118 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>106</v>
-      </c>
-      <c r="B18" s="26" t="n">
+        <v>109</v>
+      </c>
+      <c r="B18" s="34" t="n">
         <f aca="false">B$4*Supuestos!$B$43</f>
         <v>162</v>
       </c>
-      <c r="C18" s="26" t="n">
+      <c r="C18" s="34" t="n">
         <f aca="false">C$4*Supuestos!$B$43</f>
         <v>405</v>
       </c>
-      <c r="D18" s="26" t="n">
+      <c r="D18" s="34" t="n">
         <f aca="false">D$4*Supuestos!$B$43</f>
         <v>810</v>
       </c>
-      <c r="E18" s="26" t="n">
+      <c r="E18" s="34" t="n">
         <f aca="false">E$4*Supuestos!$B$43</f>
         <v>1620</v>
       </c>
-      <c r="F18" s="26" t="n">
+      <c r="F18" s="34" t="n">
         <f aca="false">F$4*Supuestos!$B$43</f>
         <v>4050</v>
       </c>
-      <c r="G18" s="26" t="n">
+      <c r="G18" s="34" t="n">
         <f aca="false">G$4*Supuestos!$B$43</f>
         <v>16200</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="B19" s="26" t="n">
+        <v>88</v>
+      </c>
+      <c r="B19" s="34" t="n">
         <f aca="false">IF(B$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>49</v>
       </c>
-      <c r="C19" s="26" t="n">
+      <c r="C19" s="34" t="n">
         <f aca="false">IF(C$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>49</v>
       </c>
-      <c r="D19" s="26" t="n">
+      <c r="D19" s="34" t="n">
         <f aca="false">IF(D$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="E19" s="26" t="n">
+      <c r="E19" s="34" t="n">
         <f aca="false">IF(E$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="F19" s="26" t="n">
+      <c r="F19" s="34" t="n">
         <f aca="false">IF(F$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
-      <c r="G19" s="26" t="n">
+      <c r="G19" s="34" t="n">
         <f aca="false">IF(G$4&gt;=Supuestos!$B$27,Supuestos!$B$28,Supuestos!$B$26)</f>
         <v>249</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>107</v>
-      </c>
-      <c r="B20" s="26" t="n">
+        <v>110</v>
+      </c>
+      <c r="B20" s="34" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="C20" s="26" t="n">
+        <v>35</v>
+      </c>
+      <c r="C20" s="34" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="D20" s="26" t="n">
+        <v>35</v>
+      </c>
+      <c r="D20" s="34" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="E20" s="26" t="n">
+        <v>35</v>
+      </c>
+      <c r="E20" s="34" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="F20" s="26" t="n">
+        <v>35</v>
+      </c>
+      <c r="F20" s="34" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
-      </c>
-      <c r="G20" s="26" t="n">
+        <v>35</v>
+      </c>
+      <c r="G20" s="34" t="n">
         <f aca="false">Supuestos!$B$25+Supuestos!$B$29+Supuestos!$B$30+Supuestos!$B$31</f>
-        <v>260</v>
+        <v>35</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B21" s="26" t="n">
+        <v>90</v>
+      </c>
+      <c r="B21" s="34" t="n">
         <f aca="false">SUM(B18:B20)</f>
-        <v>471</v>
-      </c>
-      <c r="C21" s="26" t="n">
+        <v>246</v>
+      </c>
+      <c r="C21" s="34" t="n">
         <f aca="false">SUM(C18:C20)</f>
-        <v>714</v>
-      </c>
-      <c r="D21" s="26" t="n">
+        <v>489</v>
+      </c>
+      <c r="D21" s="34" t="n">
         <f aca="false">SUM(D18:D20)</f>
-        <v>1319</v>
-      </c>
-      <c r="E21" s="26" t="n">
+        <v>1094</v>
+      </c>
+      <c r="E21" s="34" t="n">
         <f aca="false">SUM(E18:E20)</f>
-        <v>2129</v>
-      </c>
-      <c r="F21" s="26" t="n">
+        <v>1904</v>
+      </c>
+      <c r="F21" s="34" t="n">
         <f aca="false">SUM(F18:F20)</f>
-        <v>4559</v>
-      </c>
-      <c r="G21" s="26" t="n">
+        <v>4334</v>
+      </c>
+      <c r="G21" s="34" t="n">
         <f aca="false">SUM(G18:G20)</f>
-        <v>16709</v>
+        <v>16484</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2652,87 +2756,87 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="B23" s="24" t="n">
+        <v>91</v>
+      </c>
+      <c r="B23" s="36" t="n">
         <f aca="false">B15-B21</f>
-        <v>2229</v>
-      </c>
-      <c r="C23" s="24" t="n">
+        <v>2454</v>
+      </c>
+      <c r="C23" s="36" t="n">
         <f aca="false">C15-C21</f>
-        <v>6036</v>
-      </c>
-      <c r="D23" s="24" t="n">
+        <v>6261</v>
+      </c>
+      <c r="D23" s="36" t="n">
         <f aca="false">D15-D21</f>
-        <v>12181</v>
-      </c>
-      <c r="E23" s="24" t="n">
+        <v>12406</v>
+      </c>
+      <c r="E23" s="36" t="n">
         <f aca="false">E15-E21</f>
-        <v>24871</v>
-      </c>
-      <c r="F23" s="24" t="n">
+        <v>25096</v>
+      </c>
+      <c r="F23" s="36" t="n">
         <f aca="false">F15-F21</f>
-        <v>62941</v>
-      </c>
-      <c r="G23" s="24" t="n">
+        <v>63166</v>
+      </c>
+      <c r="G23" s="36" t="n">
         <f aca="false">G15-G21</f>
-        <v>253291</v>
+        <v>253516</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A24" s="3" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="B24" s="17" t="n">
         <f aca="false">IF(B15=0,0,B23/B15)</f>
-        <v>0.825555555555556</v>
+        <v>0.908888888888889</v>
       </c>
       <c r="C24" s="17" t="n">
         <f aca="false">IF(C15=0,0,C23/C15)</f>
-        <v>0.894222222222222</v>
+        <v>0.927555555555556</v>
       </c>
       <c r="D24" s="17" t="n">
         <f aca="false">IF(D15=0,0,D23/D15)</f>
-        <v>0.902296296296296</v>
+        <v>0.918962962962963</v>
       </c>
       <c r="E24" s="17" t="n">
         <f aca="false">IF(E15=0,0,E23/E15)</f>
-        <v>0.921148148148148</v>
+        <v>0.929481481481482</v>
       </c>
       <c r="F24" s="17" t="n">
         <f aca="false">IF(F15=0,0,F23/F15)</f>
-        <v>0.932459259259259</v>
+        <v>0.935792592592593</v>
       </c>
       <c r="G24" s="17" t="n">
         <f aca="false">IF(G15=0,0,G23/G15)</f>
-        <v>0.938114814814815</v>
+        <v>0.938948148148148</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>91</v>
-      </c>
-      <c r="B25" s="26" t="n">
+        <v>93</v>
+      </c>
+      <c r="B25" s="34" t="n">
         <f aca="false">IF(B$4=0,0,B15/B$4)</f>
         <v>270</v>
       </c>
-      <c r="C25" s="26" t="n">
+      <c r="C25" s="34" t="n">
         <f aca="false">IF(C$4=0,0,C15/C$4)</f>
         <v>270</v>
       </c>
-      <c r="D25" s="26" t="n">
+      <c r="D25" s="34" t="n">
         <f aca="false">IF(D$4=0,0,D15/D$4)</f>
         <v>270</v>
       </c>
-      <c r="E25" s="26" t="n">
+      <c r="E25" s="34" t="n">
         <f aca="false">IF(E$4=0,0,E15/E$4)</f>
         <v>270</v>
       </c>
-      <c r="F25" s="26" t="n">
+      <c r="F25" s="34" t="n">
         <f aca="false">IF(F$4=0,0,F15/F$4)</f>
         <v>270</v>
       </c>
-      <c r="G25" s="26" t="n">
+      <c r="G25" s="34" t="n">
         <f aca="false">IF(G$4=0,0,G15/G$4)</f>
         <v>270</v>
       </c>
@@ -2748,7 +2852,7 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B27" s="3"/>
       <c r="C27" s="3"/>
@@ -2759,7 +2863,7 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B28" s="17" t="n">
         <f aca="false">Supuestos!$B$8</f>
@@ -2788,7 +2892,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B29" s="17" t="n">
         <f aca="false">-Supuestos!$B$42</f>
@@ -2817,7 +2921,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="3" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B30" s="17" t="n">
         <f aca="false">-MAX(0,Supuestos!$B$8-Supuestos!$B$42)*Supuestos!$B$18</f>
@@ -2846,65 +2950,65 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B31" s="20" t="n">
+        <v>116</v>
+      </c>
+      <c r="B31" s="37" t="n">
         <f aca="false">B28+B29+B30</f>
         <v>-0.26</v>
       </c>
-      <c r="C31" s="20" t="n">
+      <c r="C31" s="37" t="n">
         <f aca="false">C28+C29+C30</f>
         <v>-0.26</v>
       </c>
-      <c r="D31" s="20" t="n">
+      <c r="D31" s="37" t="n">
         <f aca="false">D28+D29+D30</f>
         <v>-0.26</v>
       </c>
-      <c r="E31" s="20" t="n">
+      <c r="E31" s="37" t="n">
         <f aca="false">E28+E29+E30</f>
         <v>-0.26</v>
       </c>
-      <c r="F31" s="20" t="n">
+      <c r="F31" s="37" t="n">
         <f aca="false">F28+F29+F30</f>
         <v>-0.26</v>
       </c>
-      <c r="G31" s="20" t="n">
+      <c r="G31" s="37" t="n">
         <f aca="false">G28+G29+G30</f>
         <v>-0.26</v>
       </c>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B32" s="20" t="n">
+        <v>117</v>
+      </c>
+      <c r="B32" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="C32" s="20" t="n">
+      <c r="C32" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="D32" s="20" t="n">
+      <c r="D32" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="E32" s="20" t="n">
+      <c r="E32" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="F32" s="20" t="n">
+      <c r="F32" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="G32" s="20" t="n">
+      <c r="G32" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$41-MAX(0,Supuestos!$B$8-Supuestos!$B$41)*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="3" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B33" s="17" t="n">
         <f aca="false">Supuestos!$B$42</f>
@@ -2956,7 +3060,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -2967,7 +3071,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -2987,7 +3091,7 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="B4" s="6" t="n">
         <v>0.2</v>
@@ -3012,27 +3116,27 @@
       <c r="A5" s="8" t="n">
         <v>-0.1</v>
       </c>
-      <c r="B5" s="21" t="n">
+      <c r="B5" s="38" t="n">
         <f aca="false">$A5-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.22</v>
       </c>
-      <c r="C5" s="21" t="n">
+      <c r="C5" s="38" t="n">
         <f aca="false">$A5-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.34</v>
       </c>
-      <c r="D5" s="21" t="n">
+      <c r="D5" s="38" t="n">
         <f aca="false">$A5-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.46</v>
       </c>
-      <c r="E5" s="21" t="n">
+      <c r="E5" s="38" t="n">
         <f aca="false">$A5-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.58</v>
       </c>
-      <c r="F5" s="21" t="n">
+      <c r="F5" s="38" t="n">
         <f aca="false">$A5-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.7</v>
       </c>
-      <c r="G5" s="21" t="n">
+      <c r="G5" s="38" t="n">
         <f aca="false">$A5-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A5-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-1</v>
       </c>
@@ -3041,27 +3145,27 @@
       <c r="A6" s="8" t="n">
         <v>0</v>
       </c>
-      <c r="B6" s="21" t="n">
+      <c r="B6" s="38" t="n">
         <f aca="false">$A6-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.12</v>
       </c>
-      <c r="C6" s="21" t="n">
+      <c r="C6" s="38" t="n">
         <f aca="false">$A6-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.24</v>
       </c>
-      <c r="D6" s="21" t="n">
+      <c r="D6" s="38" t="n">
         <f aca="false">$A6-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.36</v>
       </c>
-      <c r="E6" s="21" t="n">
+      <c r="E6" s="38" t="n">
         <f aca="false">$A6-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.48</v>
       </c>
-      <c r="F6" s="21" t="n">
+      <c r="F6" s="38" t="n">
         <f aca="false">$A6-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.6</v>
       </c>
-      <c r="G6" s="21" t="n">
+      <c r="G6" s="38" t="n">
         <f aca="false">$A6-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A6-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.9</v>
       </c>
@@ -3070,27 +3174,27 @@
       <c r="A7" s="8" t="n">
         <v>0.05</v>
       </c>
-      <c r="B7" s="21" t="n">
+      <c r="B7" s="38" t="n">
         <f aca="false">$A7-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.07</v>
       </c>
-      <c r="C7" s="21" t="n">
+      <c r="C7" s="38" t="n">
         <f aca="false">$A7-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.19</v>
       </c>
-      <c r="D7" s="21" t="n">
+      <c r="D7" s="38" t="n">
         <f aca="false">$A7-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.31</v>
       </c>
-      <c r="E7" s="21" t="n">
+      <c r="E7" s="38" t="n">
         <f aca="false">$A7-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.43</v>
       </c>
-      <c r="F7" s="21" t="n">
+      <c r="F7" s="38" t="n">
         <f aca="false">$A7-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.55</v>
       </c>
-      <c r="G7" s="21" t="n">
+      <c r="G7" s="38" t="n">
         <f aca="false">$A7-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A7-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.85</v>
       </c>
@@ -3099,27 +3203,27 @@
       <c r="A8" s="8" t="n">
         <v>0.1</v>
       </c>
-      <c r="B8" s="21" t="n">
+      <c r="B8" s="38" t="n">
         <f aca="false">$A8-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.02</v>
       </c>
-      <c r="C8" s="21" t="n">
+      <c r="C8" s="38" t="n">
         <f aca="false">$A8-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.14</v>
       </c>
-      <c r="D8" s="21" t="n">
+      <c r="D8" s="38" t="n">
         <f aca="false">$A8-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.26</v>
       </c>
-      <c r="E8" s="21" t="n">
+      <c r="E8" s="38" t="n">
         <f aca="false">$A8-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.38</v>
       </c>
-      <c r="F8" s="21" t="n">
+      <c r="F8" s="38" t="n">
         <f aca="false">$A8-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.5</v>
       </c>
-      <c r="G8" s="21" t="n">
+      <c r="G8" s="38" t="n">
         <f aca="false">$A8-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A8-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.8</v>
       </c>
@@ -3128,27 +3232,27 @@
       <c r="A9" s="8" t="n">
         <v>0.2</v>
       </c>
-      <c r="B9" s="21" t="n">
+      <c r="B9" s="38" t="n">
         <f aca="false">$A9-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.072</v>
       </c>
-      <c r="C9" s="21" t="n">
+      <c r="C9" s="38" t="n">
         <f aca="false">$A9-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.04</v>
       </c>
-      <c r="D9" s="21" t="n">
+      <c r="D9" s="38" t="n">
         <f aca="false">$A9-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.16</v>
       </c>
-      <c r="E9" s="21" t="n">
+      <c r="E9" s="38" t="n">
         <f aca="false">$A9-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.28</v>
       </c>
-      <c r="F9" s="21" t="n">
+      <c r="F9" s="38" t="n">
         <f aca="false">$A9-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.4</v>
       </c>
-      <c r="G9" s="21" t="n">
+      <c r="G9" s="38" t="n">
         <f aca="false">$A9-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A9-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.7</v>
       </c>
@@ -3157,27 +3261,27 @@
       <c r="A10" s="8" t="n">
         <v>0.3</v>
       </c>
-      <c r="B10" s="21" t="n">
+      <c r="B10" s="38" t="n">
         <f aca="false">$A10-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.162</v>
       </c>
-      <c r="C10" s="21" t="n">
+      <c r="C10" s="38" t="n">
         <f aca="false">$A10-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.054</v>
       </c>
-      <c r="D10" s="21" t="n">
+      <c r="D10" s="38" t="n">
         <f aca="false">$A10-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.06</v>
       </c>
-      <c r="E10" s="21" t="n">
+      <c r="E10" s="38" t="n">
         <f aca="false">$A10-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.18</v>
       </c>
-      <c r="F10" s="21" t="n">
+      <c r="F10" s="38" t="n">
         <f aca="false">$A10-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.3</v>
       </c>
-      <c r="G10" s="21" t="n">
+      <c r="G10" s="38" t="n">
         <f aca="false">$A10-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A10-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.6</v>
       </c>
@@ -3186,27 +3290,27 @@
       <c r="A11" s="8" t="n">
         <v>0.5</v>
       </c>
-      <c r="B11" s="21" t="n">
+      <c r="B11" s="38" t="n">
         <f aca="false">$A11-(B$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(B$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.342</v>
       </c>
-      <c r="C11" s="21" t="n">
+      <c r="C11" s="38" t="n">
         <f aca="false">$A11-(C$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(C$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.234</v>
       </c>
-      <c r="D11" s="21" t="n">
+      <c r="D11" s="38" t="n">
         <f aca="false">$A11-(D$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(D$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.126</v>
       </c>
-      <c r="E11" s="21" t="n">
+      <c r="E11" s="38" t="n">
         <f aca="false">$A11-(E$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(E$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>0.018</v>
       </c>
-      <c r="F11" s="21" t="n">
+      <c r="F11" s="38" t="n">
         <f aca="false">$A11-(F$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(F$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.1</v>
       </c>
-      <c r="G11" s="21" t="n">
+      <c r="G11" s="38" t="n">
         <f aca="false">$A11-(G$4*Supuestos!$B$7*Supuestos!$B$17)-MAX(0,$A11-(G$4*Supuestos!$B$7*Supuestos!$B$17))*Supuestos!$B$18</f>
         <v>-0.4</v>
       </c>
@@ -3222,7 +3326,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="10" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
@@ -3233,237 +3337,237 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3"/>
-      <c r="B14" s="28" t="n">
+      <c r="B14" s="39" t="n">
         <f aca="false">B$4</f>
         <v>0.2</v>
       </c>
-      <c r="C14" s="28" t="n">
+      <c r="C14" s="39" t="n">
         <f aca="false">C$4</f>
         <v>0.4</v>
       </c>
-      <c r="D14" s="28" t="n">
+      <c r="D14" s="39" t="n">
         <f aca="false">D$4</f>
         <v>0.6</v>
       </c>
-      <c r="E14" s="28" t="n">
+      <c r="E14" s="39" t="n">
         <f aca="false">E$4</f>
         <v>0.8</v>
       </c>
-      <c r="F14" s="28" t="n">
+      <c r="F14" s="39" t="n">
         <f aca="false">F$4</f>
         <v>1</v>
       </c>
-      <c r="G14" s="28" t="n">
+      <c r="G14" s="39" t="n">
         <f aca="false">G$4</f>
         <v>1.5</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A15" s="21" t="n">
+      <c r="A15" s="38" t="n">
         <f aca="false">$A5</f>
         <v>-0.1</v>
       </c>
-      <c r="B15" s="21" t="n">
+      <c r="B15" s="38" t="n">
         <f aca="false">$A15-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.16</v>
       </c>
-      <c r="C15" s="21" t="n">
+      <c r="C15" s="38" t="n">
         <f aca="false">$A15-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.22</v>
       </c>
-      <c r="D15" s="21" t="n">
+      <c r="D15" s="38" t="n">
         <f aca="false">$A15-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.28</v>
       </c>
-      <c r="E15" s="21" t="n">
+      <c r="E15" s="38" t="n">
         <f aca="false">$A15-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.34</v>
       </c>
-      <c r="F15" s="21" t="n">
+      <c r="F15" s="38" t="n">
         <f aca="false">$A15-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.4</v>
       </c>
-      <c r="G15" s="21" t="n">
+      <c r="G15" s="38" t="n">
         <f aca="false">$A15-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A15-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.55</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A16" s="21" t="n">
+      <c r="A16" s="38" t="n">
         <f aca="false">$A6</f>
         <v>0</v>
       </c>
-      <c r="B16" s="21" t="n">
+      <c r="B16" s="38" t="n">
         <f aca="false">$A16-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.06</v>
       </c>
-      <c r="C16" s="21" t="n">
+      <c r="C16" s="38" t="n">
         <f aca="false">$A16-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.12</v>
       </c>
-      <c r="D16" s="21" t="n">
+      <c r="D16" s="38" t="n">
         <f aca="false">$A16-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.18</v>
       </c>
-      <c r="E16" s="21" t="n">
+      <c r="E16" s="38" t="n">
         <f aca="false">$A16-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.24</v>
       </c>
-      <c r="F16" s="21" t="n">
+      <c r="F16" s="38" t="n">
         <f aca="false">$A16-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.3</v>
       </c>
-      <c r="G16" s="21" t="n">
+      <c r="G16" s="38" t="n">
         <f aca="false">$A16-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A16-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.45</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="38" t="n">
         <f aca="false">$A7</f>
         <v>0.05</v>
       </c>
-      <c r="B17" s="21" t="n">
+      <c r="B17" s="38" t="n">
         <f aca="false">$A17-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.01</v>
       </c>
-      <c r="C17" s="21" t="n">
+      <c r="C17" s="38" t="n">
         <f aca="false">$A17-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.07</v>
       </c>
-      <c r="D17" s="21" t="n">
+      <c r="D17" s="38" t="n">
         <f aca="false">$A17-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.13</v>
       </c>
-      <c r="E17" s="21" t="n">
+      <c r="E17" s="38" t="n">
         <f aca="false">$A17-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.19</v>
       </c>
-      <c r="F17" s="21" t="n">
+      <c r="F17" s="38" t="n">
         <f aca="false">$A17-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.25</v>
       </c>
-      <c r="G17" s="21" t="n">
+      <c r="G17" s="38" t="n">
         <f aca="false">$A17-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A17-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.4</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="38" t="n">
         <f aca="false">$A8</f>
         <v>0.1</v>
       </c>
-      <c r="B18" s="21" t="n">
+      <c r="B18" s="38" t="n">
         <f aca="false">$A18-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.04</v>
       </c>
-      <c r="C18" s="21" t="n">
+      <c r="C18" s="38" t="n">
         <f aca="false">$A18-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.02</v>
       </c>
-      <c r="D18" s="21" t="n">
+      <c r="D18" s="38" t="n">
         <f aca="false">$A18-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.08</v>
       </c>
-      <c r="E18" s="21" t="n">
+      <c r="E18" s="38" t="n">
         <f aca="false">$A18-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.14</v>
       </c>
-      <c r="F18" s="21" t="n">
+      <c r="F18" s="38" t="n">
         <f aca="false">$A18-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.2</v>
       </c>
-      <c r="G18" s="21" t="n">
+      <c r="G18" s="38" t="n">
         <f aca="false">$A18-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A18-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.35</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A19" s="21" t="n">
+      <c r="A19" s="38" t="n">
         <f aca="false">$A9</f>
         <v>0.2</v>
       </c>
-      <c r="B19" s="21" t="n">
+      <c r="B19" s="38" t="n">
         <f aca="false">$A19-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.14</v>
       </c>
-      <c r="C19" s="21" t="n">
+      <c r="C19" s="38" t="n">
         <f aca="false">$A19-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.08</v>
       </c>
-      <c r="D19" s="21" t="n">
+      <c r="D19" s="38" t="n">
         <f aca="false">$A19-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.02</v>
       </c>
-      <c r="E19" s="21" t="n">
+      <c r="E19" s="38" t="n">
         <f aca="false">$A19-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.04</v>
       </c>
-      <c r="F19" s="21" t="n">
+      <c r="F19" s="38" t="n">
         <f aca="false">$A19-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.1</v>
       </c>
-      <c r="G19" s="21" t="n">
+      <c r="G19" s="38" t="n">
         <f aca="false">$A19-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A19-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.25</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A20" s="21" t="n">
+      <c r="A20" s="38" t="n">
         <f aca="false">$A10</f>
         <v>0.3</v>
       </c>
-      <c r="B20" s="21" t="n">
+      <c r="B20" s="38" t="n">
         <f aca="false">$A20-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.24</v>
       </c>
-      <c r="C20" s="21" t="n">
+      <c r="C20" s="38" t="n">
         <f aca="false">$A20-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.18</v>
       </c>
-      <c r="D20" s="21" t="n">
+      <c r="D20" s="38" t="n">
         <f aca="false">$A20-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.12</v>
       </c>
-      <c r="E20" s="21" t="n">
+      <c r="E20" s="38" t="n">
         <f aca="false">$A20-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.06</v>
       </c>
-      <c r="F20" s="21" t="n">
+      <c r="F20" s="38" t="n">
         <f aca="false">$A20-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0</v>
       </c>
-      <c r="G20" s="21" t="n">
+      <c r="G20" s="38" t="n">
         <f aca="false">$A20-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A20-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>-0.15</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A21" s="21" t="n">
+      <c r="A21" s="38" t="n">
         <f aca="false">$A11</f>
         <v>0.5</v>
       </c>
-      <c r="B21" s="21" t="n">
+      <c r="B21" s="38" t="n">
         <f aca="false">$A21-(B$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(B$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.44</v>
       </c>
-      <c r="C21" s="21" t="n">
+      <c r="C21" s="38" t="n">
         <f aca="false">$A21-(C$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(C$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.38</v>
       </c>
-      <c r="D21" s="21" t="n">
+      <c r="D21" s="38" t="n">
         <f aca="false">$A21-(D$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(D$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.32</v>
       </c>
-      <c r="E21" s="21" t="n">
+      <c r="E21" s="38" t="n">
         <f aca="false">$A21-(E$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(E$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.26</v>
       </c>
-      <c r="F21" s="21" t="n">
+      <c r="F21" s="38" t="n">
         <f aca="false">$A21-(F$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(F$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.2</v>
       </c>
-      <c r="G21" s="21" t="n">
+      <c r="G21" s="38" t="n">
         <f aca="false">$A21-(G$4*Supuestos!$B$7*Supuestos!$B$15)-MAX(0,$A21-(G$4*Supuestos!$B$7*Supuestos!$B$15))*Supuestos!$B$16</f>
         <v>0.05</v>
       </c>
@@ -3509,7 +3613,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3517,7 +3621,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3532,20 +3636,20 @@
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10"/>
       <c r="B4" s="10" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C4" s="10" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D4" s="10" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B5" s="29" t="n">
+      <c r="B5" s="40" t="n">
         <f aca="false">Supuestos!$B$17</f>
         <v>0.02</v>
       </c>
@@ -3558,9 +3662,9 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>125</v>
-      </c>
-      <c r="B6" s="29" t="n">
+        <v>128</v>
+      </c>
+      <c r="B6" s="40" t="n">
         <f aca="false">Supuestos!$B$18</f>
         <v>0.1</v>
       </c>
@@ -3573,9 +3677,9 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>126</v>
-      </c>
-      <c r="B7" s="29" t="n">
+        <v>129</v>
+      </c>
+      <c r="B7" s="40" t="n">
         <f aca="false">Supuestos!$B$15</f>
         <v>0.01</v>
       </c>
@@ -3588,9 +3692,9 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>127</v>
-      </c>
-      <c r="B8" s="29" t="n">
+        <v>130</v>
+      </c>
+      <c r="B8" s="40" t="n">
         <f aca="false">Supuestos!$B$16</f>
         <v>0</v>
       </c>
@@ -3603,7 +3707,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B9" s="12" t="n">
         <v>0</v>
@@ -3616,8 +3720,8 @@
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="30" t="s">
-        <v>129</v>
+      <c r="A10" s="41" t="s">
+        <v>132</v>
       </c>
       <c r="B10" s="3"/>
       <c r="C10" s="3"/>
@@ -3631,7 +3735,7 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
@@ -3639,187 +3743,187 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="B13" s="23" t="n">
+        <v>134</v>
+      </c>
+      <c r="B13" s="42" t="n">
         <f aca="false">1000*Supuestos!$B$8</f>
         <v>100</v>
       </c>
-      <c r="C13" s="23" t="n">
+      <c r="C13" s="42" t="n">
         <f aca="false">1000*Supuestos!$B$8</f>
         <v>100</v>
       </c>
-      <c r="D13" s="23" t="n">
+      <c r="D13" s="42" t="n">
         <f aca="false">1000*Supuestos!$B$8</f>
         <v>100</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="B14" s="23" t="n">
+        <v>135</v>
+      </c>
+      <c r="B14" s="42" t="n">
         <f aca="false">1000*Supuestos!$B$40*B$5</f>
         <v>360</v>
       </c>
-      <c r="C14" s="23" t="n">
+      <c r="C14" s="42" t="n">
         <f aca="false">1000*Supuestos!$B$40*C$5</f>
         <v>45</v>
       </c>
-      <c r="D14" s="23" t="n">
+      <c r="D14" s="42" t="n">
         <f aca="false">1000*Supuestos!$B$40*D$5</f>
         <v>0</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="B15" s="23" t="n">
+        <v>136</v>
+      </c>
+      <c r="B15" s="42" t="n">
         <f aca="false">B13-B14</f>
         <v>-260</v>
       </c>
-      <c r="C15" s="23" t="n">
+      <c r="C15" s="42" t="n">
         <f aca="false">C13-C14</f>
         <v>55</v>
       </c>
-      <c r="D15" s="23" t="n">
+      <c r="D15" s="42" t="n">
         <f aca="false">D13-D14</f>
         <v>100</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="B16" s="23" t="n">
+        <v>137</v>
+      </c>
+      <c r="B16" s="42" t="n">
         <f aca="false">MAX(0,B15)*B$6</f>
         <v>0</v>
       </c>
-      <c r="C16" s="23" t="n">
+      <c r="C16" s="42" t="n">
         <f aca="false">MAX(0,C15)*C$6</f>
         <v>11</v>
       </c>
-      <c r="D16" s="23" t="n">
+      <c r="D16" s="42" t="n">
         <f aca="false">MAX(0,D15)*D$6</f>
         <v>25</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="B17" s="23" t="n">
+        <v>138</v>
+      </c>
+      <c r="B17" s="42" t="n">
         <f aca="false">B$9</f>
         <v>0</v>
       </c>
-      <c r="C17" s="23" t="n">
+      <c r="C17" s="42" t="n">
         <f aca="false">C$9</f>
         <v>0</v>
       </c>
-      <c r="D17" s="23" t="n">
+      <c r="D17" s="42" t="n">
         <f aca="false">D$9</f>
         <v>0</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B18" s="24" t="n">
+        <v>139</v>
+      </c>
+      <c r="B18" s="36" t="n">
         <f aca="false">B15-B16-B17</f>
         <v>-260</v>
       </c>
-      <c r="C18" s="24" t="n">
+      <c r="C18" s="36" t="n">
         <f aca="false">C15-C16-C17</f>
         <v>44</v>
       </c>
-      <c r="D18" s="24" t="n">
+      <c r="D18" s="36" t="n">
         <f aca="false">D15-D16-D17</f>
         <v>75</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="B19" s="20" t="n">
+        <v>140</v>
+      </c>
+      <c r="B19" s="37" t="n">
         <f aca="false">B18/1000</f>
         <v>-0.26</v>
       </c>
-      <c r="C19" s="20" t="n">
+      <c r="C19" s="37" t="n">
         <f aca="false">C18/1000</f>
         <v>0.044</v>
       </c>
-      <c r="D19" s="20" t="n">
+      <c r="D19" s="37" t="n">
         <f aca="false">D18/1000</f>
         <v>0.075</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="B20" s="24" t="n">
+        <v>141</v>
+      </c>
+      <c r="B20" s="36" t="n">
         <f aca="false">B14+B16+B17</f>
         <v>360</v>
       </c>
-      <c r="C20" s="24" t="n">
+      <c r="C20" s="36" t="n">
         <f aca="false">C14+C16+C17</f>
         <v>56</v>
       </c>
-      <c r="D20" s="24" t="n">
+      <c r="D20" s="36" t="n">
         <f aca="false">D14+D16+D17</f>
         <v>25</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="B21" s="23" t="n">
+        <v>142</v>
+      </c>
+      <c r="B21" s="42" t="n">
         <f aca="false">Supuestos!$B$43</f>
         <v>16.2</v>
       </c>
-      <c r="C21" s="23" t="n">
+      <c r="C21" s="42" t="n">
         <f aca="false">Supuestos!$B$43</f>
         <v>16.2</v>
       </c>
-      <c r="D21" s="23" t="n">
+      <c r="D21" s="42" t="n">
         <f aca="false">Supuestos!$B$43</f>
         <v>16.2</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A22" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="B22" s="23" t="n">
+        <v>143</v>
+      </c>
+      <c r="B22" s="42" t="n">
         <f aca="false">B20-B21</f>
         <v>343.8</v>
       </c>
-      <c r="C22" s="23" t="n">
+      <c r="C22" s="42" t="n">
         <f aca="false">C20-C21</f>
         <v>39.8</v>
       </c>
-      <c r="D22" s="23" t="n">
+      <c r="D22" s="42" t="n">
         <f aca="false">D20-D21</f>
         <v>8.8</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="B23" s="21" t="n">
+        <v>144</v>
+      </c>
+      <c r="B23" s="38" t="n">
         <f aca="false">B14/1000</f>
         <v>0.36</v>
       </c>
-      <c r="C23" s="21" t="n">
+      <c r="C23" s="38" t="n">
         <f aca="false">C14/1000</f>
         <v>0.045</v>
       </c>
-      <c r="D23" s="21" t="n">
+      <c r="D23" s="38" t="n">
         <f aca="false">D14/1000</f>
         <v>0</v>
       </c>
@@ -3832,7 +3936,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
@@ -3840,68 +3944,68 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="B26" s="23" t="n">
+        <v>134</v>
+      </c>
+      <c r="B26" s="42" t="n">
         <f aca="false">1000*-0.1</f>
         <v>-100</v>
       </c>
-      <c r="C26" s="23" t="n">
+      <c r="C26" s="42" t="n">
         <f aca="false">1000*-0.1</f>
         <v>-100</v>
       </c>
-      <c r="D26" s="23" t="n">
+      <c r="D26" s="42" t="n">
         <f aca="false">1000*-0.1</f>
         <v>-100</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="B27" s="23" t="n">
+        <v>135</v>
+      </c>
+      <c r="B27" s="42" t="n">
         <f aca="false">1000*Supuestos!$B$40*B$5</f>
         <v>360</v>
       </c>
-      <c r="C27" s="23" t="n">
+      <c r="C27" s="42" t="n">
         <f aca="false">1000*Supuestos!$B$40*C$5</f>
         <v>45</v>
       </c>
-      <c r="D27" s="23" t="n">
+      <c r="D27" s="42" t="n">
         <f aca="false">1000*Supuestos!$B$40*D$5</f>
         <v>0</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="B28" s="24" t="n">
+        <v>139</v>
+      </c>
+      <c r="B28" s="36" t="n">
         <f aca="false">B26-B27-B$9</f>
         <v>-460</v>
       </c>
-      <c r="C28" s="24" t="n">
+      <c r="C28" s="36" t="n">
         <f aca="false">C26-C27-C$9</f>
         <v>-145</v>
       </c>
-      <c r="D28" s="24" t="n">
+      <c r="D28" s="36" t="n">
         <f aca="false">D26-D27-D$9</f>
         <v>-100</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="B29" s="24" t="n">
+        <v>141</v>
+      </c>
+      <c r="B29" s="36" t="n">
         <f aca="false">B27+B$9</f>
         <v>360</v>
       </c>
-      <c r="C29" s="24" t="n">
+      <c r="C29" s="36" t="n">
         <f aca="false">C27+C$9</f>
         <v>45</v>
       </c>
-      <c r="D29" s="24" t="n">
+      <c r="D29" s="36" t="n">
         <f aca="false">D27+D$9</f>
         <v>0</v>
       </c>
@@ -3913,8 +4017,8 @@
       <c r="D30" s="3"/>
     </row>
     <row r="31" customFormat="false" ht="42" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A31" s="31" t="s">
-        <v>143</v>
+      <c r="A31" s="43" t="s">
+        <v>146</v>
       </c>
       <c r="B31" s="3"/>
       <c r="C31" s="3"/>
@@ -3945,7 +4049,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
@@ -3956,7 +4060,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3976,348 +4080,348 @@
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="10" t="s">
-        <v>79</v>
-      </c>
-      <c r="B4" s="32" t="n">
+        <v>81</v>
+      </c>
+      <c r="B4" s="44" t="n">
         <f aca="false">Escenarios!B4</f>
         <v>10</v>
       </c>
-      <c r="C4" s="32" t="n">
+      <c r="C4" s="44" t="n">
         <f aca="false">Escenarios!C4</f>
         <v>25</v>
       </c>
-      <c r="D4" s="32" t="n">
+      <c r="D4" s="44" t="n">
         <f aca="false">Escenarios!D4</f>
         <v>50</v>
       </c>
-      <c r="E4" s="32" t="n">
+      <c r="E4" s="44" t="n">
         <f aca="false">Escenarios!E4</f>
         <v>100</v>
       </c>
-      <c r="F4" s="32" t="n">
+      <c r="F4" s="44" t="n">
         <f aca="false">Escenarios!F4</f>
         <v>250</v>
       </c>
-      <c r="G4" s="32" t="n">
+      <c r="G4" s="44" t="n">
         <f aca="false">Escenarios!G4</f>
         <v>1000</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>96</v>
-      </c>
-      <c r="B5" s="23" t="n">
+        <v>99</v>
+      </c>
+      <c r="B5" s="42" t="n">
         <f aca="false">B$4*Supuestos!$B$34</f>
         <v>10000</v>
       </c>
-      <c r="C5" s="23" t="n">
+      <c r="C5" s="42" t="n">
         <f aca="false">C$4*Supuestos!$B$34</f>
         <v>25000</v>
       </c>
-      <c r="D5" s="23" t="n">
+      <c r="D5" s="42" t="n">
         <f aca="false">D$4*Supuestos!$B$34</f>
         <v>50000</v>
       </c>
-      <c r="E5" s="23" t="n">
+      <c r="E5" s="42" t="n">
         <f aca="false">E$4*Supuestos!$B$34</f>
         <v>100000</v>
       </c>
-      <c r="F5" s="23" t="n">
+      <c r="F5" s="42" t="n">
         <f aca="false">F$4*Supuestos!$B$34</f>
         <v>250000</v>
       </c>
-      <c r="G5" s="23" t="n">
+      <c r="G5" s="42" t="n">
         <f aca="false">G$4*Supuestos!$B$34</f>
         <v>1000000</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="3" t="s">
-        <v>97</v>
-      </c>
-      <c r="B6" s="23" t="n">
+        <v>100</v>
+      </c>
+      <c r="B6" s="42" t="n">
         <f aca="false">B5*Supuestos!$B$35</f>
         <v>5000</v>
       </c>
-      <c r="C6" s="23" t="n">
+      <c r="C6" s="42" t="n">
         <f aca="false">C5*Supuestos!$B$35</f>
         <v>12500</v>
       </c>
-      <c r="D6" s="23" t="n">
+      <c r="D6" s="42" t="n">
         <f aca="false">D5*Supuestos!$B$35</f>
         <v>25000</v>
       </c>
-      <c r="E6" s="23" t="n">
+      <c r="E6" s="42" t="n">
         <f aca="false">E5*Supuestos!$B$35</f>
         <v>50000</v>
       </c>
-      <c r="F6" s="23" t="n">
+      <c r="F6" s="42" t="n">
         <f aca="false">F5*Supuestos!$B$35</f>
         <v>125000</v>
       </c>
-      <c r="G6" s="23" t="n">
+      <c r="G6" s="42" t="n">
         <f aca="false">G5*Supuestos!$B$35</f>
         <v>500000</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B7" s="23" t="n">
+        <v>101</v>
+      </c>
+      <c r="B7" s="42" t="n">
         <f aca="false">B5-B6</f>
         <v>5000</v>
       </c>
-      <c r="C7" s="23" t="n">
+      <c r="C7" s="42" t="n">
         <f aca="false">C5-C6</f>
         <v>12500</v>
       </c>
-      <c r="D7" s="23" t="n">
+      <c r="D7" s="42" t="n">
         <f aca="false">D5-D6</f>
         <v>25000</v>
       </c>
-      <c r="E7" s="23" t="n">
+      <c r="E7" s="42" t="n">
         <f aca="false">E5-E6</f>
         <v>50000</v>
       </c>
-      <c r="F7" s="23" t="n">
+      <c r="F7" s="42" t="n">
         <f aca="false">F5-F6</f>
         <v>125000</v>
       </c>
-      <c r="G7" s="23" t="n">
+      <c r="G7" s="42" t="n">
         <f aca="false">G5-G6</f>
         <v>500000</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="B8" s="23" t="n">
+        <v>149</v>
+      </c>
+      <c r="B8" s="42" t="n">
         <f aca="false">(B6*Alternativas!$C$7+B7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>450</v>
       </c>
-      <c r="C8" s="23" t="n">
+      <c r="C8" s="42" t="n">
         <f aca="false">(C6*Alternativas!$C$7+C7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>1125</v>
       </c>
-      <c r="D8" s="23" t="n">
+      <c r="D8" s="42" t="n">
         <f aca="false">(D6*Alternativas!$C$7+D7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>2250</v>
       </c>
-      <c r="E8" s="23" t="n">
+      <c r="E8" s="42" t="n">
         <f aca="false">(E6*Alternativas!$C$7+E7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>4500</v>
       </c>
-      <c r="F8" s="23" t="n">
+      <c r="F8" s="42" t="n">
         <f aca="false">(F6*Alternativas!$C$7+F7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>11250</v>
       </c>
-      <c r="G8" s="23" t="n">
+      <c r="G8" s="42" t="n">
         <f aca="false">(G6*Alternativas!$C$7+G7*Alternativas!$C$5)*Supuestos!$B$40</f>
         <v>45000</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="3" t="s">
-        <v>147</v>
-      </c>
-      <c r="B9" s="23" t="n">
+        <v>150</v>
+      </c>
+      <c r="B9" s="42" t="n">
         <f aca="false">B7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+B6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>82.5</v>
       </c>
-      <c r="C9" s="23" t="n">
+      <c r="C9" s="42" t="n">
         <f aca="false">C7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+C6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>206.25</v>
       </c>
-      <c r="D9" s="23" t="n">
+      <c r="D9" s="42" t="n">
         <f aca="false">D7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+D6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>412.5</v>
       </c>
-      <c r="E9" s="23" t="n">
+      <c r="E9" s="42" t="n">
         <f aca="false">E7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+E6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>825</v>
       </c>
-      <c r="F9" s="23" t="n">
+      <c r="F9" s="42" t="n">
         <f aca="false">F7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+F6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>2062.5</v>
       </c>
-      <c r="G9" s="23" t="n">
+      <c r="G9" s="42" t="n">
         <f aca="false">G7*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6+G6*MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>8250</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="3" t="s">
-        <v>148</v>
-      </c>
-      <c r="B10" s="23" t="n">
+        <v>151</v>
+      </c>
+      <c r="B10" s="42" t="n">
         <f aca="false">B$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
-      <c r="C10" s="23" t="n">
+      <c r="C10" s="42" t="n">
         <f aca="false">C$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
-      <c r="D10" s="23" t="n">
+      <c r="D10" s="42" t="n">
         <f aca="false">D$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
-      <c r="E10" s="23" t="n">
+      <c r="E10" s="42" t="n">
         <f aca="false">E$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
-      <c r="F10" s="23" t="n">
+      <c r="F10" s="42" t="n">
         <f aca="false">F$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
-      <c r="G10" s="23" t="n">
+      <c r="G10" s="42" t="n">
         <f aca="false">G$4*Alternativas!$C$9</f>
         <v>0</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="3" t="s">
-        <v>84</v>
-      </c>
-      <c r="B11" s="23" t="n">
+        <v>86</v>
+      </c>
+      <c r="B11" s="42" t="n">
         <f aca="false">SUM(B8:B10)</f>
         <v>532.5</v>
       </c>
-      <c r="C11" s="23" t="n">
+      <c r="C11" s="42" t="n">
         <f aca="false">SUM(C8:C10)</f>
         <v>1331.25</v>
       </c>
-      <c r="D11" s="23" t="n">
+      <c r="D11" s="42" t="n">
         <f aca="false">SUM(D8:D10)</f>
         <v>2662.5</v>
       </c>
-      <c r="E11" s="23" t="n">
+      <c r="E11" s="42" t="n">
         <f aca="false">SUM(E8:E10)</f>
         <v>5325</v>
       </c>
-      <c r="F11" s="23" t="n">
+      <c r="F11" s="42" t="n">
         <f aca="false">SUM(F8:F10)</f>
         <v>13312.5</v>
       </c>
-      <c r="G11" s="23" t="n">
+      <c r="G11" s="42" t="n">
         <f aca="false">SUM(G8:G10)</f>
         <v>53250</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="B12" s="23" t="n">
+        <v>90</v>
+      </c>
+      <c r="B12" s="42" t="n">
         <f aca="false">Escenarios!B21</f>
-        <v>471</v>
-      </c>
-      <c r="C12" s="23" t="n">
+        <v>246</v>
+      </c>
+      <c r="C12" s="42" t="n">
         <f aca="false">Escenarios!C21</f>
-        <v>714</v>
-      </c>
-      <c r="D12" s="23" t="n">
+        <v>489</v>
+      </c>
+      <c r="D12" s="42" t="n">
         <f aca="false">Escenarios!D21</f>
-        <v>1319</v>
-      </c>
-      <c r="E12" s="23" t="n">
+        <v>1094</v>
+      </c>
+      <c r="E12" s="42" t="n">
         <f aca="false">Escenarios!E21</f>
-        <v>2129</v>
-      </c>
-      <c r="F12" s="23" t="n">
+        <v>1904</v>
+      </c>
+      <c r="F12" s="42" t="n">
         <f aca="false">Escenarios!F21</f>
-        <v>4559</v>
-      </c>
-      <c r="G12" s="23" t="n">
+        <v>4334</v>
+      </c>
+      <c r="G12" s="42" t="n">
         <f aca="false">Escenarios!G21</f>
-        <v>16709</v>
+        <v>16484</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="B13" s="24" t="n">
+        <v>91</v>
+      </c>
+      <c r="B13" s="36" t="n">
         <f aca="false">B11-B12</f>
-        <v>61.5000000000001</v>
-      </c>
-      <c r="C13" s="24" t="n">
+        <v>286.5</v>
+      </c>
+      <c r="C13" s="36" t="n">
         <f aca="false">C11-C12</f>
-        <v>617.25</v>
-      </c>
-      <c r="D13" s="24" t="n">
+        <v>842.25</v>
+      </c>
+      <c r="D13" s="36" t="n">
         <f aca="false">D11-D12</f>
-        <v>1343.5</v>
-      </c>
-      <c r="E13" s="24" t="n">
+        <v>1568.5</v>
+      </c>
+      <c r="E13" s="36" t="n">
         <f aca="false">E11-E12</f>
-        <v>3196</v>
-      </c>
-      <c r="F13" s="24" t="n">
+        <v>3421</v>
+      </c>
+      <c r="F13" s="36" t="n">
         <f aca="false">F11-F12</f>
-        <v>8753.5</v>
-      </c>
-      <c r="G13" s="24" t="n">
+        <v>8978.5</v>
+      </c>
+      <c r="G13" s="36" t="n">
         <f aca="false">G11-G12</f>
-        <v>36541</v>
+        <v>36766</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="B14" s="20" t="n">
+        <v>116</v>
+      </c>
+      <c r="B14" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
-      <c r="C14" s="20" t="n">
+      <c r="C14" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
-      <c r="D14" s="20" t="n">
+      <c r="D14" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
-      <c r="F14" s="20" t="n">
+      <c r="F14" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
-      <c r="G14" s="20" t="n">
+      <c r="G14" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$5)*Alternativas!$C$6</f>
         <v>0.044</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="B15" s="20" t="n">
+        <v>117</v>
+      </c>
+      <c r="B15" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>
-      <c r="C15" s="20" t="n">
+      <c r="C15" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>
-      <c r="D15" s="20" t="n">
+      <c r="D15" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>
-      <c r="E15" s="20" t="n">
+      <c r="E15" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>
-      <c r="F15" s="20" t="n">
+      <c r="F15" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>
-      <c r="G15" s="20" t="n">
+      <c r="G15" s="37" t="n">
         <f aca="false">Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7-MAX(0,Supuestos!$B$8-Supuestos!$B$40*Alternativas!$C$7)*Alternativas!$C$8</f>
         <v>0.0495</v>
       </c>

</xml_diff>